<commit_message>
Fase 4: cierre de resultados 2026-08-28
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,8 +501,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -549,8 +547,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -597,8 +593,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -645,8 +639,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -693,8 +685,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -741,8 +731,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -789,8 +777,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -837,8 +823,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -885,8 +869,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -933,8 +915,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -981,8 +961,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1029,8 +1007,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1077,8 +1053,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1125,8 +1099,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1173,8 +1145,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1221,8 +1191,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1269,8 +1237,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1317,8 +1283,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1365,8 +1329,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1413,8 +1375,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1461,8 +1421,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1509,8 +1467,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1557,8 +1513,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1605,8 +1559,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1653,8 +1605,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1701,8 +1651,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
       <c r="G27" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1749,8 +1697,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1797,8 +1743,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1845,8 +1789,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1893,8 +1835,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1941,8 +1881,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -1989,8 +1927,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -2037,8 +1973,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -2059,6 +1993,2838 @@
         <v>0</v>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Akron Tolyatti vs CSKA Moscow</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CSKA Moscow</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Al Riyadh vs Neom SC</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Neom SC</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Al Fayha vs Abha</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Al Fayha</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>VfL Bochum vs VfL Osnabruck</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>VfL Bochum</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Racing Santander vs Elche</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Racing Santander</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>AC Horsens vs Viborg FF</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Viborg FF</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Austria Lustenau vs WSG Swarovski Tirol</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Austria Lustenau</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>FC Groningen vs Fortuna Sittard</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>FC Groningen</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Stade Laval vs Grenoble</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Stade Laval</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Montpellier vs Boulogne</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Montpellier</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Rodez Aveyron vs Pau</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Rodez Aveyron</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>FC Volendam vs FC Dordrecht</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>FC Volendam</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Jong Ajax vs Helmond Sport</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Jong Ajax</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Jong AZ vs MVV Maastricht</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Jong AZ</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>TOP Oss vs Jong FC Utrecht</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>TOP Oss</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>0</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Roda JC Kerkrade vs NAC Breda</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>NAC Breda</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>RKC Waalwijk vs Jong PSV</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>RKC Waalwijk</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Al Khaleej vs Al Hilal</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Al Hilal</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Al Nassr vs Al Taawoun</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Al Nassr</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Clermont Foot vs Sochaux</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Clermont Foot</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>AS Nancy Lorraine vs Dunkerque</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>AS Nancy Lorraine</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>FC Den Bosch vs Vitesse</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bayern Munich vs VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Cremonese vs Modena</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Cremonese</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Lille vs Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>0</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>AC Milan vs Venezia</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>AC Milan</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>0</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Racing Genk vs Waasland-Beveren</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Racing Genk</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>AFC Fylde vs Forest Green Rovers</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Forest Green Rovers</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Aldershot Town vs Harrogate Town</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Harrogate Town</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Altrincham vs FC Halifax Town</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Altrincham</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Barrow vs Yeovil Town</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Barrow</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Gateshead vs Sutton United</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Sutton United</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Hartlepool United vs Eastleigh</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Hartlepool United</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>AFC Hornchurch vs Woking</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>AFC Hornchurch</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Scunthorpe United vs Solihull Moors</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Scunthorpe United</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Southend United vs Kidderminster Harriers</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Southend United</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>0</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Tamworth vs Worthing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Tamworth</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr"/>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Crystal Palace vs Manchester City</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Wrexham vs Birmingham City</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Wrexham</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Sportivo Luqueño vs Rubio Ñú</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Sportivo Luqueño</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Tenerife vs Sporting Gijón</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Tenerife</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="n">
+        <v>0</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Beira Mar vs União Lamas</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Beira Mar</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="n">
+        <v>0</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Rio Ave vs Sporting CP</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr"/>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Alavés vs Villarreal</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Villarreal</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Comerciantes Unidos vs FC Cajamarca</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Comerciantes Unidos</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" t="n">
+        <v>0</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Mushuc Runa vs Delfín</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" t="n">
+        <v>0</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0</v>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Unión (Santa Fe) vs Sarmiento (Junín)</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Unión (Santa Fe)</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
+        <v>0</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Montevideo Wanderers vs Central Español Fútbol Club</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Montevideo Wanderers</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="n">
+        <v>0</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>CD Municipal Limeño vs Isidro Metapán</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>CD Municipal Limeño</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" t="n">
+        <v>0</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Goiás vs São Bernardo</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Goiás</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="n">
+        <v>0</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Charlotte Independence vs AV Alta FC</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Charlotte Independence</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" t="n">
+        <v>0</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Náutico vs Athletic</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Náutico</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="n">
+        <v>0</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0</v>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Novorizontino vs Sport</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Novorizontino</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>0</v>
+      </c>
+      <c r="J87" t="n">
+        <v>0</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0</v>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Técnico Universitario vs Deportivo Cuenca</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Técnico Universitario</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>0</v>
+      </c>
+      <c r="J88" t="n">
+        <v>0</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Boca Juniors vs Lanús</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Boca Juniors</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" t="n">
+        <v>0</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Necaxa vs Cruz Azul</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Cruz Azul</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" t="n">
+        <v>0</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Gimnasia y Tiro (Salta) vs Chacarita Juniors</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Gimnasia y Tiro (Salta)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Sporting San José vs Inter de San Carlos</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Sporting San José</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Suchitepequez vs Cobán Imperial</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Suchitepequez</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -2075,7 +4841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2119,6 +4885,22 @@
       </c>
       <c r="E2" t="n">
         <v>111</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>59</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-01
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L284"/>
+  <dimension ref="A1:L328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9655,8 +9655,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr"/>
-      <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -9703,8 +9701,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -9751,8 +9747,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr"/>
-      <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -9799,8 +9793,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr"/>
-      <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -9847,8 +9839,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr"/>
       <c r="G205" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -9895,8 +9885,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -9943,8 +9931,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr"/>
       <c r="G207" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -9991,8 +9977,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
       <c r="G208" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10039,8 +10023,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr"/>
-      <c r="F209" t="inlineStr"/>
       <c r="G209" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10087,8 +10069,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr"/>
-      <c r="F210" t="inlineStr"/>
       <c r="G210" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10135,8 +10115,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr"/>
-      <c r="F211" t="inlineStr"/>
       <c r="G211" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10183,8 +10161,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10231,8 +10207,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10279,8 +10253,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
       <c r="G214" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10327,8 +10299,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10375,8 +10345,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr"/>
-      <c r="F216" t="inlineStr"/>
       <c r="G216" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10423,8 +10391,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr"/>
-      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10471,8 +10437,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr"/>
-      <c r="F218" t="inlineStr"/>
       <c r="G218" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10519,8 +10483,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
       <c r="G219" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10567,8 +10529,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10615,8 +10575,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr"/>
       <c r="G221" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10663,8 +10621,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr"/>
-      <c r="F222" t="inlineStr"/>
       <c r="G222" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10711,8 +10667,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr"/>
-      <c r="F223" t="inlineStr"/>
       <c r="G223" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10759,8 +10713,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
-      <c r="F224" t="inlineStr"/>
       <c r="G224" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10807,8 +10759,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr"/>
-      <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10855,8 +10805,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E226" t="inlineStr"/>
-      <c r="F226" t="inlineStr"/>
       <c r="G226" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10903,8 +10851,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr"/>
       <c r="G227" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10951,8 +10897,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -10999,8 +10943,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr"/>
       <c r="G229" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11047,8 +10989,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E230" t="inlineStr"/>
-      <c r="F230" t="inlineStr"/>
       <c r="G230" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11095,8 +11035,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E231" t="inlineStr"/>
-      <c r="F231" t="inlineStr"/>
       <c r="G231" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11143,8 +11081,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr"/>
-      <c r="F232" t="inlineStr"/>
       <c r="G232" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11191,8 +11127,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr"/>
-      <c r="F233" t="inlineStr"/>
       <c r="G233" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11239,8 +11173,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E234" t="inlineStr"/>
-      <c r="F234" t="inlineStr"/>
       <c r="G234" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11287,8 +11219,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
       <c r="G235" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11335,8 +11265,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
-      <c r="F236" t="inlineStr"/>
       <c r="G236" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11383,8 +11311,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr"/>
-      <c r="F237" t="inlineStr"/>
       <c r="G237" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11431,8 +11357,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E238" t="inlineStr"/>
-      <c r="F238" t="inlineStr"/>
       <c r="G238" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11479,8 +11403,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr"/>
-      <c r="F239" t="inlineStr"/>
       <c r="G239" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11527,8 +11449,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr"/>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11575,8 +11495,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E241" t="inlineStr"/>
-      <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11623,8 +11541,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E242" t="inlineStr"/>
-      <c r="F242" t="inlineStr"/>
       <c r="G242" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11671,8 +11587,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E243" t="inlineStr"/>
-      <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11719,8 +11633,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E244" t="inlineStr"/>
-      <c r="F244" t="inlineStr"/>
       <c r="G244" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11767,8 +11679,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E245" t="inlineStr"/>
-      <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11815,8 +11725,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E246" t="inlineStr"/>
-      <c r="F246" t="inlineStr"/>
       <c r="G246" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11863,8 +11771,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E247" t="inlineStr"/>
-      <c r="F247" t="inlineStr"/>
       <c r="G247" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11911,8 +11817,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E248" t="inlineStr"/>
-      <c r="F248" t="inlineStr"/>
       <c r="G248" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -11959,8 +11863,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E249" t="inlineStr"/>
-      <c r="F249" t="inlineStr"/>
       <c r="G249" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12007,8 +11909,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E250" t="inlineStr"/>
-      <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12055,8 +11955,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E251" t="inlineStr"/>
-      <c r="F251" t="inlineStr"/>
       <c r="G251" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12103,8 +12001,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E252" t="inlineStr"/>
-      <c r="F252" t="inlineStr"/>
       <c r="G252" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12151,8 +12047,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E253" t="inlineStr"/>
-      <c r="F253" t="inlineStr"/>
       <c r="G253" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12199,8 +12093,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr"/>
-      <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12247,8 +12139,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr"/>
-      <c r="F255" t="inlineStr"/>
       <c r="G255" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12295,8 +12185,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr"/>
-      <c r="F256" t="inlineStr"/>
       <c r="G256" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12343,8 +12231,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E257" t="inlineStr"/>
-      <c r="F257" t="inlineStr"/>
       <c r="G257" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12391,8 +12277,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E258" t="inlineStr"/>
-      <c r="F258" t="inlineStr"/>
       <c r="G258" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12439,8 +12323,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E259" t="inlineStr"/>
-      <c r="F259" t="inlineStr"/>
       <c r="G259" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12487,8 +12369,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E260" t="inlineStr"/>
-      <c r="F260" t="inlineStr"/>
       <c r="G260" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12535,8 +12415,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E261" t="inlineStr"/>
-      <c r="F261" t="inlineStr"/>
       <c r="G261" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12583,8 +12461,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E262" t="inlineStr"/>
-      <c r="F262" t="inlineStr"/>
       <c r="G262" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12631,8 +12507,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E263" t="inlineStr"/>
-      <c r="F263" t="inlineStr"/>
       <c r="G263" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12679,8 +12553,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E264" t="inlineStr"/>
-      <c r="F264" t="inlineStr"/>
       <c r="G264" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12727,8 +12599,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E265" t="inlineStr"/>
-      <c r="F265" t="inlineStr"/>
       <c r="G265" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12775,8 +12645,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E266" t="inlineStr"/>
-      <c r="F266" t="inlineStr"/>
       <c r="G266" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12823,8 +12691,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E267" t="inlineStr"/>
-      <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12871,8 +12737,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E268" t="inlineStr"/>
-      <c r="F268" t="inlineStr"/>
       <c r="G268" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12919,8 +12783,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E269" t="inlineStr"/>
-      <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -12967,8 +12829,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E270" t="inlineStr"/>
-      <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13015,8 +12875,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E271" t="inlineStr"/>
-      <c r="F271" t="inlineStr"/>
       <c r="G271" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13063,8 +12921,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr"/>
-      <c r="F272" t="inlineStr"/>
       <c r="G272" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13111,8 +12967,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E273" t="inlineStr"/>
-      <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13159,8 +13013,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E274" t="inlineStr"/>
-      <c r="F274" t="inlineStr"/>
       <c r="G274" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13207,8 +13059,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E275" t="inlineStr"/>
-      <c r="F275" t="inlineStr"/>
       <c r="G275" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13255,8 +13105,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E276" t="inlineStr"/>
-      <c r="F276" t="inlineStr"/>
       <c r="G276" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13303,8 +13151,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E277" t="inlineStr"/>
-      <c r="F277" t="inlineStr"/>
       <c r="G277" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13351,8 +13197,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E278" t="inlineStr"/>
-      <c r="F278" t="inlineStr"/>
       <c r="G278" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13399,8 +13243,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E279" t="inlineStr"/>
-      <c r="F279" t="inlineStr"/>
       <c r="G279" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13447,8 +13289,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E280" t="inlineStr"/>
-      <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13495,8 +13335,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E281" t="inlineStr"/>
-      <c r="F281" t="inlineStr"/>
       <c r="G281" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13543,8 +13381,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E282" t="inlineStr"/>
-      <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13591,8 +13427,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E283" t="inlineStr"/>
-      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13639,8 +13473,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E284" t="inlineStr"/>
-      <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -13661,6 +13493,2118 @@
         <v>0</v>
       </c>
       <c r="L284" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Persib vs Manila Digger</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Persib</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr"/>
+      <c r="F285" t="inlineStr"/>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I285" t="n">
+        <v>0</v>
+      </c>
+      <c r="J285" t="n">
+        <v>0</v>
+      </c>
+      <c r="K285" t="n">
+        <v>0</v>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Boston United vs AFC Hornchurch</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Boston United</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr"/>
+      <c r="F286" t="inlineStr"/>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I286" t="n">
+        <v>0</v>
+      </c>
+      <c r="J286" t="n">
+        <v>0</v>
+      </c>
+      <c r="K286" t="n">
+        <v>0</v>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Carlisle United vs Scunthorpe United</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Carlisle United</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr"/>
+      <c r="F287" t="inlineStr"/>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I287" t="n">
+        <v>0</v>
+      </c>
+      <c r="J287" t="n">
+        <v>0</v>
+      </c>
+      <c r="K287" t="n">
+        <v>0</v>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Eastleigh vs Aldershot Town</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Eastleigh</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr"/>
+      <c r="F288" t="inlineStr"/>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I288" t="n">
+        <v>0</v>
+      </c>
+      <c r="J288" t="n">
+        <v>0</v>
+      </c>
+      <c r="K288" t="n">
+        <v>0</v>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Forest Green Rovers vs Altrincham</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Forest Green Rovers</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr"/>
+      <c r="F289" t="inlineStr"/>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I289" t="n">
+        <v>0</v>
+      </c>
+      <c r="J289" t="n">
+        <v>0</v>
+      </c>
+      <c r="K289" t="n">
+        <v>0</v>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Harrogate Town vs Gateshead</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Harrogate Town</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr"/>
+      <c r="F290" t="inlineStr"/>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I290" t="n">
+        <v>0</v>
+      </c>
+      <c r="J290" t="n">
+        <v>0</v>
+      </c>
+      <c r="K290" t="n">
+        <v>0</v>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Kidderminster Harriers vs Barrow</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Barrow</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr"/>
+      <c r="F291" t="inlineStr"/>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I291" t="n">
+        <v>0</v>
+      </c>
+      <c r="J291" t="n">
+        <v>0</v>
+      </c>
+      <c r="K291" t="n">
+        <v>0</v>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Solihull Moors vs AFC Fylde</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>Solihull Moors</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr"/>
+      <c r="F292" t="inlineStr"/>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I292" t="n">
+        <v>0</v>
+      </c>
+      <c r="J292" t="n">
+        <v>0</v>
+      </c>
+      <c r="K292" t="n">
+        <v>0</v>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Sutton United vs Wealdstone</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Sutton United</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr"/>
+      <c r="F293" t="inlineStr"/>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I293" t="n">
+        <v>0</v>
+      </c>
+      <c r="J293" t="n">
+        <v>0</v>
+      </c>
+      <c r="K293" t="n">
+        <v>0</v>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Woking vs Southend United</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Southend United</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr"/>
+      <c r="F294" t="inlineStr"/>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I294" t="n">
+        <v>0</v>
+      </c>
+      <c r="J294" t="n">
+        <v>0</v>
+      </c>
+      <c r="K294" t="n">
+        <v>0</v>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Worthing vs Boreham Wood</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Boreham Wood</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr"/>
+      <c r="F295" t="inlineStr"/>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I295" t="n">
+        <v>0</v>
+      </c>
+      <c r="J295" t="n">
+        <v>0</v>
+      </c>
+      <c r="K295" t="n">
+        <v>0</v>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Lecce vs AS Roma</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>AS Roma</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr"/>
+      <c r="F296" t="inlineStr"/>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I296" t="n">
+        <v>0</v>
+      </c>
+      <c r="J296" t="n">
+        <v>0</v>
+      </c>
+      <c r="K296" t="n">
+        <v>0</v>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Levadiakos vs Panathinaikos</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>Panathinaikos</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr"/>
+      <c r="F297" t="inlineStr"/>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I297" t="n">
+        <v>0</v>
+      </c>
+      <c r="J297" t="n">
+        <v>0</v>
+      </c>
+      <c r="K297" t="n">
+        <v>0</v>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>F.C. København vs Sønderjyske Fodbold</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>F.C. København</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr"/>
+      <c r="F298" t="inlineStr"/>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I298" t="n">
+        <v>0</v>
+      </c>
+      <c r="J298" t="n">
+        <v>0</v>
+      </c>
+      <c r="K298" t="n">
+        <v>0</v>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Djurgården vs Mjällby AIF</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Djurgården</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr"/>
+      <c r="F299" t="inlineStr"/>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I299" t="n">
+        <v>0</v>
+      </c>
+      <c r="J299" t="n">
+        <v>0</v>
+      </c>
+      <c r="K299" t="n">
+        <v>0</v>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>GAIS vs IF Brommapojkarna</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>GAIS</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr"/>
+      <c r="F300" t="inlineStr"/>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I300" t="n">
+        <v>0</v>
+      </c>
+      <c r="J300" t="n">
+        <v>0</v>
+      </c>
+      <c r="K300" t="n">
+        <v>0</v>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>IK Sirius vs Malmö FF</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>IK Sirius</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr"/>
+      <c r="F301" t="inlineStr"/>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I301" t="n">
+        <v>0</v>
+      </c>
+      <c r="J301" t="n">
+        <v>0</v>
+      </c>
+      <c r="K301" t="n">
+        <v>0</v>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Burgos vs Real Sociedad II</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr"/>
+      <c r="F302" t="inlineStr"/>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I302" t="n">
+        <v>0</v>
+      </c>
+      <c r="J302" t="n">
+        <v>0</v>
+      </c>
+      <c r="K302" t="n">
+        <v>0</v>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Osasuna vs Getafe</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Osasuna</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr"/>
+      <c r="F303" t="inlineStr"/>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I303" t="n">
+        <v>0</v>
+      </c>
+      <c r="J303" t="n">
+        <v>0</v>
+      </c>
+      <c r="K303" t="n">
+        <v>0</v>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Jong AZ vs Jong FC Utrecht</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Jong AZ</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr"/>
+      <c r="F304" t="inlineStr"/>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I304" t="n">
+        <v>0</v>
+      </c>
+      <c r="J304" t="n">
+        <v>0</v>
+      </c>
+      <c r="K304" t="n">
+        <v>0</v>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Jong PSV vs Jong Ajax</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Jong PSV</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr"/>
+      <c r="F305" t="inlineStr"/>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I305" t="n">
+        <v>0</v>
+      </c>
+      <c r="J305" t="n">
+        <v>0</v>
+      </c>
+      <c r="K305" t="n">
+        <v>0</v>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Amed SFK vs Trabzonspor</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Trabzonspor</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr"/>
+      <c r="F306" t="inlineStr"/>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>0</v>
+      </c>
+      <c r="J306" t="n">
+        <v>0</v>
+      </c>
+      <c r="K306" t="n">
+        <v>0</v>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Besiktas vs Çorum FK</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Besiktas</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr"/>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>6-2</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>0</v>
+      </c>
+      <c r="J307" t="n">
+        <v>0</v>
+      </c>
+      <c r="K307" t="n">
+        <v>0</v>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Racing (Montevideo) vs Albion FC</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Racing (Montevideo)</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr"/>
+      <c r="F308" t="inlineStr"/>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>0</v>
+      </c>
+      <c r="J308" t="n">
+        <v>0</v>
+      </c>
+      <c r="K308" t="n">
+        <v>0</v>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Atalanta vs Bologna</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr"/>
+      <c r="F309" t="inlineStr"/>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>0</v>
+      </c>
+      <c r="J309" t="n">
+        <v>0</v>
+      </c>
+      <c r="K309" t="n">
+        <v>0</v>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Dijon FCO vs Saint-Étienne</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Saint-Étienne</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr"/>
+      <c r="F310" t="inlineStr"/>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>0</v>
+      </c>
+      <c r="J310" t="n">
+        <v>0</v>
+      </c>
+      <c r="K310" t="n">
+        <v>0</v>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Aston Villa vs Arsenal</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr"/>
+      <c r="F311" t="inlineStr"/>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>0</v>
+      </c>
+      <c r="J311" t="n">
+        <v>0</v>
+      </c>
+      <c r="K311" t="n">
+        <v>0</v>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>San Antonio Bulo Bulo vs Guabirá</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>San Antonio Bulo Bulo</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr"/>
+      <c r="F312" t="inlineStr"/>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>0</v>
+      </c>
+      <c r="J312" t="n">
+        <v>0</v>
+      </c>
+      <c r="K312" t="n">
+        <v>0</v>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Benfica vs Estoril</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr"/>
+      <c r="F313" t="inlineStr"/>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>0</v>
+      </c>
+      <c r="J313" t="n">
+        <v>0</v>
+      </c>
+      <c r="K313" t="n">
+        <v>0</v>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Braga vs Vitória de Guimaraes</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr"/>
+      <c r="F314" t="inlineStr"/>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J314" t="n">
+        <v>0</v>
+      </c>
+      <c r="K314" t="n">
+        <v>0</v>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Barcelona vs Rayo Vallecano</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr"/>
+      <c r="F315" t="inlineStr"/>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>5-2</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I315" t="n">
+        <v>0</v>
+      </c>
+      <c r="J315" t="n">
+        <v>0</v>
+      </c>
+      <c r="K315" t="n">
+        <v>0</v>
+      </c>
+      <c r="L315" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Defensa y Justicia vs Platense</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Defensa y Justicia</t>
+        </is>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr"/>
+      <c r="F316" t="inlineStr"/>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I316" t="n">
+        <v>0</v>
+      </c>
+      <c r="J316" t="n">
+        <v>0</v>
+      </c>
+      <c r="K316" t="n">
+        <v>0</v>
+      </c>
+      <c r="L316" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Newell's Old Boys</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr"/>
+      <c r="F317" t="inlineStr"/>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I317" t="n">
+        <v>0</v>
+      </c>
+      <c r="J317" t="n">
+        <v>0</v>
+      </c>
+      <c r="K317" t="n">
+        <v>0</v>
+      </c>
+      <c r="L317" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Comunicaciones vs Deportivo Merlo</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr"/>
+      <c r="F318" t="inlineStr"/>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I318" t="n">
+        <v>0</v>
+      </c>
+      <c r="J318" t="n">
+        <v>0</v>
+      </c>
+      <c r="K318" t="n">
+        <v>0</v>
+      </c>
+      <c r="L318" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Los Andes vs Acassuso</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Los Andes</t>
+        </is>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr"/>
+      <c r="F319" t="inlineStr"/>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I319" t="n">
+        <v>0</v>
+      </c>
+      <c r="J319" t="n">
+        <v>0</v>
+      </c>
+      <c r="K319" t="n">
+        <v>0</v>
+      </c>
+      <c r="L319" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Unión La Calera vs La Serena</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Unión La Calera</t>
+        </is>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr"/>
+      <c r="F320" t="inlineStr"/>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I320" t="n">
+        <v>0</v>
+      </c>
+      <c r="J320" t="n">
+        <v>0</v>
+      </c>
+      <c r="K320" t="n">
+        <v>0</v>
+      </c>
+      <c r="L320" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>UCV FC vs Rayo Zuliano</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>UCV FC</t>
+        </is>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr"/>
+      <c r="F321" t="inlineStr"/>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I321" t="n">
+        <v>0</v>
+      </c>
+      <c r="J321" t="n">
+        <v>0</v>
+      </c>
+      <c r="K321" t="n">
+        <v>0</v>
+      </c>
+      <c r="L321" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Fortaleza vs Operário PR</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr"/>
+      <c r="F322" t="inlineStr"/>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I322" t="n">
+        <v>0</v>
+      </c>
+      <c r="J322" t="n">
+        <v>0</v>
+      </c>
+      <c r="K322" t="n">
+        <v>0</v>
+      </c>
+      <c r="L322" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Remo vs Coritiba</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Remo</t>
+        </is>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr"/>
+      <c r="F323" t="inlineStr"/>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I323" t="n">
+        <v>0</v>
+      </c>
+      <c r="J323" t="n">
+        <v>0</v>
+      </c>
+      <c r="K323" t="n">
+        <v>0</v>
+      </c>
+      <c r="L323" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Deportivo Pasto vs Deportivo Pereira</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Deportivo Pasto</t>
+        </is>
+      </c>
+      <c r="D324" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr"/>
+      <c r="F324" t="inlineStr"/>
+      <c r="G324" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H324" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I324" t="n">
+        <v>0</v>
+      </c>
+      <c r="J324" t="n">
+        <v>0</v>
+      </c>
+      <c r="K324" t="n">
+        <v>0</v>
+      </c>
+      <c r="L324" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Academia Puerto Cabello vs Anzoátegui FC</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>Academia Puerto Cabello</t>
+        </is>
+      </c>
+      <c r="D325" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr"/>
+      <c r="F325" t="inlineStr"/>
+      <c r="G325" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H325" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I325" t="n">
+        <v>0</v>
+      </c>
+      <c r="J325" t="n">
+        <v>0</v>
+      </c>
+      <c r="K325" t="n">
+        <v>0</v>
+      </c>
+      <c r="L325" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Instituto (Córdoba) vs San Lorenzo</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Instituto (Córdoba)</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr"/>
+      <c r="F326" t="inlineStr"/>
+      <c r="G326" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I326" t="n">
+        <v>0</v>
+      </c>
+      <c r="J326" t="n">
+        <v>0</v>
+      </c>
+      <c r="K326" t="n">
+        <v>0</v>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Tigre vs Barracas Central</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Tigre</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr"/>
+      <c r="F327" t="inlineStr"/>
+      <c r="G327" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I327" t="n">
+        <v>0</v>
+      </c>
+      <c r="J327" t="n">
+        <v>0</v>
+      </c>
+      <c r="K327" t="n">
+        <v>0</v>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Deportes Tolima vs Cúcuta Deportivo</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Deportes Tolima</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr"/>
+      <c r="F328" t="inlineStr"/>
+      <c r="G328" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H328" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I328" t="n">
+        <v>0</v>
+      </c>
+      <c r="J328" t="n">
+        <v>0</v>
+      </c>
+      <c r="K328" t="n">
+        <v>0</v>
+      </c>
+      <c r="L328" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -13677,7 +15621,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13769,6 +15713,25 @@
       </c>
       <c r="E5" t="n">
         <v>146</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>44</v>
+      </c>
+      <c r="C6" t="n">
+        <v>33</v>
+      </c>
+      <c r="D6" t="n">
+        <v>75</v>
+      </c>
+      <c r="E6" t="n">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-02
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L328"/>
+  <dimension ref="A1:L362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13519,8 +13519,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E285" t="inlineStr"/>
-      <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -13567,8 +13565,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E286" t="inlineStr"/>
-      <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -13615,8 +13611,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E287" t="inlineStr"/>
-      <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -13663,8 +13657,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E288" t="inlineStr"/>
-      <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -13711,8 +13703,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr"/>
-      <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -13759,8 +13749,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E290" t="inlineStr"/>
-      <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -13807,8 +13795,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E291" t="inlineStr"/>
-      <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -13855,8 +13841,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr"/>
-      <c r="F292" t="inlineStr"/>
       <c r="G292" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -13903,8 +13887,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E293" t="inlineStr"/>
-      <c r="F293" t="inlineStr"/>
       <c r="G293" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -13951,8 +13933,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E294" t="inlineStr"/>
-      <c r="F294" t="inlineStr"/>
       <c r="G294" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -13999,8 +13979,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E295" t="inlineStr"/>
-      <c r="F295" t="inlineStr"/>
       <c r="G295" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -14047,8 +14025,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E296" t="inlineStr"/>
-      <c r="F296" t="inlineStr"/>
       <c r="G296" t="inlineStr">
         <is>
           <t>0-4</t>
@@ -14095,8 +14071,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E297" t="inlineStr"/>
-      <c r="F297" t="inlineStr"/>
       <c r="G297" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -14143,8 +14117,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E298" t="inlineStr"/>
-      <c r="F298" t="inlineStr"/>
       <c r="G298" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -14191,8 +14163,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E299" t="inlineStr"/>
-      <c r="F299" t="inlineStr"/>
       <c r="G299" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -14239,8 +14209,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E300" t="inlineStr"/>
-      <c r="F300" t="inlineStr"/>
       <c r="G300" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -14287,8 +14255,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E301" t="inlineStr"/>
-      <c r="F301" t="inlineStr"/>
       <c r="G301" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -14335,8 +14301,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E302" t="inlineStr"/>
-      <c r="F302" t="inlineStr"/>
       <c r="G302" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -14383,8 +14347,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E303" t="inlineStr"/>
-      <c r="F303" t="inlineStr"/>
       <c r="G303" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -14431,8 +14393,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E304" t="inlineStr"/>
-      <c r="F304" t="inlineStr"/>
       <c r="G304" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -14479,8 +14439,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E305" t="inlineStr"/>
-      <c r="F305" t="inlineStr"/>
       <c r="G305" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -14527,8 +14485,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E306" t="inlineStr"/>
-      <c r="F306" t="inlineStr"/>
       <c r="G306" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -14575,8 +14531,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E307" t="inlineStr"/>
-      <c r="F307" t="inlineStr"/>
       <c r="G307" t="inlineStr">
         <is>
           <t>6-2</t>
@@ -14623,8 +14577,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E308" t="inlineStr"/>
-      <c r="F308" t="inlineStr"/>
       <c r="G308" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -14671,8 +14623,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E309" t="inlineStr"/>
-      <c r="F309" t="inlineStr"/>
       <c r="G309" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -14719,8 +14669,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E310" t="inlineStr"/>
-      <c r="F310" t="inlineStr"/>
       <c r="G310" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -14767,8 +14715,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E311" t="inlineStr"/>
-      <c r="F311" t="inlineStr"/>
       <c r="G311" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -14815,8 +14761,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E312" t="inlineStr"/>
-      <c r="F312" t="inlineStr"/>
       <c r="G312" t="inlineStr">
         <is>
           <t>5-1</t>
@@ -14863,8 +14807,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E313" t="inlineStr"/>
-      <c r="F313" t="inlineStr"/>
       <c r="G313" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -14911,8 +14853,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E314" t="inlineStr"/>
-      <c r="F314" t="inlineStr"/>
       <c r="G314" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -14959,8 +14899,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E315" t="inlineStr"/>
-      <c r="F315" t="inlineStr"/>
       <c r="G315" t="inlineStr">
         <is>
           <t>5-2</t>
@@ -15007,8 +14945,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E316" t="inlineStr"/>
-      <c r="F316" t="inlineStr"/>
       <c r="G316" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -15055,8 +14991,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E317" t="inlineStr"/>
-      <c r="F317" t="inlineStr"/>
       <c r="G317" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -15103,8 +15037,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E318" t="inlineStr"/>
-      <c r="F318" t="inlineStr"/>
       <c r="G318" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -15151,8 +15083,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E319" t="inlineStr"/>
-      <c r="F319" t="inlineStr"/>
       <c r="G319" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -15199,8 +15129,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E320" t="inlineStr"/>
-      <c r="F320" t="inlineStr"/>
       <c r="G320" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -15247,8 +15175,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E321" t="inlineStr"/>
-      <c r="F321" t="inlineStr"/>
       <c r="G321" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -15295,8 +15221,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E322" t="inlineStr"/>
-      <c r="F322" t="inlineStr"/>
       <c r="G322" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -15343,8 +15267,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E323" t="inlineStr"/>
-      <c r="F323" t="inlineStr"/>
       <c r="G323" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -15391,8 +15313,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E324" t="inlineStr"/>
-      <c r="F324" t="inlineStr"/>
       <c r="G324" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -15439,8 +15359,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E325" t="inlineStr"/>
-      <c r="F325" t="inlineStr"/>
       <c r="G325" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -15487,8 +15405,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E326" t="inlineStr"/>
-      <c r="F326" t="inlineStr"/>
       <c r="G326" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -15535,8 +15451,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E327" t="inlineStr"/>
-      <c r="F327" t="inlineStr"/>
       <c r="G327" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -15583,8 +15497,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E328" t="inlineStr"/>
-      <c r="F328" t="inlineStr"/>
       <c r="G328" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -15605,6 +15517,1638 @@
         <v>0</v>
       </c>
       <c r="L328" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Avispa Fukuoka vs Urawa Red Diamonds</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Avispa Fukuoka</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr"/>
+      <c r="F329" t="inlineStr"/>
+      <c r="G329" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I329" t="n">
+        <v>0</v>
+      </c>
+      <c r="J329" t="n">
+        <v>0</v>
+      </c>
+      <c r="K329" t="n">
+        <v>0</v>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Cerezo Osaka vs Kashiwa Reysol</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Kashiwa Reysol</t>
+        </is>
+      </c>
+      <c r="D330" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr"/>
+      <c r="F330" t="inlineStr"/>
+      <c r="G330" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I330" t="n">
+        <v>0</v>
+      </c>
+      <c r="J330" t="n">
+        <v>0</v>
+      </c>
+      <c r="K330" t="n">
+        <v>0</v>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Machida Zelvia vs Kawasaki Frontale</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Machida Zelvia</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr"/>
+      <c r="F331" t="inlineStr"/>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I331" t="n">
+        <v>0</v>
+      </c>
+      <c r="J331" t="n">
+        <v>0</v>
+      </c>
+      <c r="K331" t="n">
+        <v>0</v>
+      </c>
+      <c r="L331" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Mito Hollyhock vs Kashima Antlers</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Kashima Antlers</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr"/>
+      <c r="F332" t="inlineStr"/>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H332" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I332" t="n">
+        <v>0</v>
+      </c>
+      <c r="J332" t="n">
+        <v>0</v>
+      </c>
+      <c r="K332" t="n">
+        <v>0</v>
+      </c>
+      <c r="L332" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Sanfrecce Hiroshima vs Nagoya Grampus</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Sanfrecce Hiroshima</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr"/>
+      <c r="F333" t="inlineStr"/>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H333" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I333" t="n">
+        <v>0</v>
+      </c>
+      <c r="J333" t="n">
+        <v>0</v>
+      </c>
+      <c r="K333" t="n">
+        <v>0</v>
+      </c>
+      <c r="L333" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Shimizu S-Pulse vs FC Tokyo</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>FC Tokyo</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr"/>
+      <c r="F334" t="inlineStr"/>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H334" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I334" t="n">
+        <v>0</v>
+      </c>
+      <c r="J334" t="n">
+        <v>0</v>
+      </c>
+      <c r="K334" t="n">
+        <v>0</v>
+      </c>
+      <c r="L334" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Tokyo Verdy 1969 vs Vissel Kobe</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Vissel Kobe</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr"/>
+      <c r="F335" t="inlineStr"/>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H335" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I335" t="n">
+        <v>0</v>
+      </c>
+      <c r="J335" t="n">
+        <v>0</v>
+      </c>
+      <c r="K335" t="n">
+        <v>0</v>
+      </c>
+      <c r="L335" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>V-Varen Nagasaki vs Gamba Osaka</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Gamba Osaka</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr"/>
+      <c r="F336" t="inlineStr"/>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H336" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I336" t="n">
+        <v>0</v>
+      </c>
+      <c r="J336" t="n">
+        <v>0</v>
+      </c>
+      <c r="K336" t="n">
+        <v>0</v>
+      </c>
+      <c r="L336" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Yokohama F. Marinos vs Kyoto Sanga</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Yokohama F. Marinos</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr"/>
+      <c r="F337" t="inlineStr"/>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H337" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I337" t="n">
+        <v>0</v>
+      </c>
+      <c r="J337" t="n">
+        <v>0</v>
+      </c>
+      <c r="K337" t="n">
+        <v>0</v>
+      </c>
+      <c r="L337" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Sassuolo vs Frosinone</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Sassuolo</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr"/>
+      <c r="F338" t="inlineStr"/>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H338" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I338" t="n">
+        <v>0</v>
+      </c>
+      <c r="J338" t="n">
+        <v>0</v>
+      </c>
+      <c r="K338" t="n">
+        <v>0</v>
+      </c>
+      <c r="L338" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Udinese vs Venezia</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Udinese</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr"/>
+      <c r="F339" t="inlineStr"/>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H339" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I339" t="n">
+        <v>0</v>
+      </c>
+      <c r="J339" t="n">
+        <v>0</v>
+      </c>
+      <c r="K339" t="n">
+        <v>0</v>
+      </c>
+      <c r="L339" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Austria Vienna vs WSG Swarovski Tirol</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Austria Vienna</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr"/>
+      <c r="F340" t="inlineStr"/>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H340" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I340" t="n">
+        <v>0</v>
+      </c>
+      <c r="J340" t="n">
+        <v>0</v>
+      </c>
+      <c r="K340" t="n">
+        <v>0</v>
+      </c>
+      <c r="L340" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>AGF vs FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr"/>
+      <c r="F341" t="inlineStr"/>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H341" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I341" t="n">
+        <v>0</v>
+      </c>
+      <c r="J341" t="n">
+        <v>0</v>
+      </c>
+      <c r="K341" t="n">
+        <v>0</v>
+      </c>
+      <c r="L341" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Sint-Truidense vs Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Union St.-Gilloise</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr"/>
+      <c r="F342" t="inlineStr"/>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H342" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I342" t="n">
+        <v>0</v>
+      </c>
+      <c r="J342" t="n">
+        <v>0</v>
+      </c>
+      <c r="K342" t="n">
+        <v>0</v>
+      </c>
+      <c r="L342" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Millwall vs Wrexham</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Millwall</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr"/>
+      <c r="F343" t="inlineStr"/>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H343" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I343" t="n">
+        <v>0</v>
+      </c>
+      <c r="J343" t="n">
+        <v>0</v>
+      </c>
+      <c r="K343" t="n">
+        <v>0</v>
+      </c>
+      <c r="L343" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Queens Park Rangers vs Cardiff City</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Queens Park Rangers</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr"/>
+      <c r="F344" t="inlineStr"/>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H344" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I344" t="n">
+        <v>0</v>
+      </c>
+      <c r="J344" t="n">
+        <v>0</v>
+      </c>
+      <c r="K344" t="n">
+        <v>0</v>
+      </c>
+      <c r="L344" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>West Bromwich Albion vs Charlton Athletic</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>West Bromwich Albion</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr"/>
+      <c r="F345" t="inlineStr"/>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I345" t="n">
+        <v>0</v>
+      </c>
+      <c r="J345" t="n">
+        <v>0</v>
+      </c>
+      <c r="K345" t="n">
+        <v>0</v>
+      </c>
+      <c r="L345" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Barnsley vs Blackpool</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Barnsley</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr"/>
+      <c r="F346" t="inlineStr"/>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I346" t="n">
+        <v>0</v>
+      </c>
+      <c r="J346" t="n">
+        <v>0</v>
+      </c>
+      <c r="K346" t="n">
+        <v>0</v>
+      </c>
+      <c r="L346" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Burton Albion vs AFC Wimbledon</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Burton Albion</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr"/>
+      <c r="F347" t="inlineStr"/>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I347" t="n">
+        <v>0</v>
+      </c>
+      <c r="J347" t="n">
+        <v>0</v>
+      </c>
+      <c r="K347" t="n">
+        <v>0</v>
+      </c>
+      <c r="L347" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Luton Town vs Stockport County</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Luton Town</t>
+        </is>
+      </c>
+      <c r="D348" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr"/>
+      <c r="F348" t="inlineStr"/>
+      <c r="G348" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H348" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I348" t="n">
+        <v>0</v>
+      </c>
+      <c r="J348" t="n">
+        <v>0</v>
+      </c>
+      <c r="K348" t="n">
+        <v>0</v>
+      </c>
+      <c r="L348" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Wigan Athletic vs Milton Keynes Dons</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Wigan Athletic</t>
+        </is>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr"/>
+      <c r="F349" t="inlineStr"/>
+      <c r="G349" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H349" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I349" t="n">
+        <v>0</v>
+      </c>
+      <c r="J349" t="n">
+        <v>0</v>
+      </c>
+      <c r="K349" t="n">
+        <v>0</v>
+      </c>
+      <c r="L349" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Celtic vs Aberdeen</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
+      <c r="D350" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr"/>
+      <c r="F350" t="inlineStr"/>
+      <c r="G350" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H350" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I350" t="n">
+        <v>0</v>
+      </c>
+      <c r="J350" t="n">
+        <v>0</v>
+      </c>
+      <c r="K350" t="n">
+        <v>0</v>
+      </c>
+      <c r="L350" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Motherwell vs Dundee United</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Motherwell</t>
+        </is>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr"/>
+      <c r="F351" t="inlineStr"/>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H351" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I351" t="n">
+        <v>0</v>
+      </c>
+      <c r="J351" t="n">
+        <v>0</v>
+      </c>
+      <c r="K351" t="n">
+        <v>0</v>
+      </c>
+      <c r="L351" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>VfL Osnabruck vs Bayern Munich</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr"/>
+      <c r="F352" t="inlineStr"/>
+      <c r="G352" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H352" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I352" t="n">
+        <v>0</v>
+      </c>
+      <c r="J352" t="n">
+        <v>0</v>
+      </c>
+      <c r="K352" t="n">
+        <v>0</v>
+      </c>
+      <c r="L352" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Reading vs Mansfield Town</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Reading</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr"/>
+      <c r="F353" t="inlineStr"/>
+      <c r="G353" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H353" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I353" t="n">
+        <v>0</v>
+      </c>
+      <c r="J353" t="n">
+        <v>0</v>
+      </c>
+      <c r="K353" t="n">
+        <v>0</v>
+      </c>
+      <c r="L353" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Falkirk vs Rangers</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Rangers</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E354" t="inlineStr"/>
+      <c r="F354" t="inlineStr"/>
+      <c r="G354" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H354" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I354" t="n">
+        <v>0</v>
+      </c>
+      <c r="J354" t="n">
+        <v>0</v>
+      </c>
+      <c r="K354" t="n">
+        <v>0</v>
+      </c>
+      <c r="L354" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Macará vs Manta F.C.</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Macará</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr"/>
+      <c r="F355" t="inlineStr"/>
+      <c r="G355" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H355" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I355" t="n">
+        <v>0</v>
+      </c>
+      <c r="J355" t="n">
+        <v>0</v>
+      </c>
+      <c r="K355" t="n">
+        <v>0</v>
+      </c>
+      <c r="L355" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Nacional Asunción vs Libertad</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Nacional Asunción</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E356" t="inlineStr"/>
+      <c r="F356" t="inlineStr"/>
+      <c r="G356" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H356" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I356" t="n">
+        <v>0</v>
+      </c>
+      <c r="J356" t="n">
+        <v>0</v>
+      </c>
+      <c r="K356" t="n">
+        <v>0</v>
+      </c>
+      <c r="L356" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Deportivo Cuenca vs Guayaquil City FC</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Deportivo Cuenca</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr"/>
+      <c r="F357" t="inlineStr"/>
+      <c r="G357" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H357" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I357" t="n">
+        <v>0</v>
+      </c>
+      <c r="J357" t="n">
+        <v>0</v>
+      </c>
+      <c r="K357" t="n">
+        <v>0</v>
+      </c>
+      <c r="L357" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Club Olimpia vs Guaraní</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Club Olimpia</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E358" t="inlineStr"/>
+      <c r="F358" t="inlineStr"/>
+      <c r="G358" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H358" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I358" t="n">
+        <v>0</v>
+      </c>
+      <c r="J358" t="n">
+        <v>0</v>
+      </c>
+      <c r="K358" t="n">
+        <v>0</v>
+      </c>
+      <c r="L358" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Coquimbo Unido vs Universidad de Concepción</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>Coquimbo Unido</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr"/>
+      <c r="F359" t="inlineStr"/>
+      <c r="G359" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H359" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I359" t="n">
+        <v>0</v>
+      </c>
+      <c r="J359" t="n">
+        <v>0</v>
+      </c>
+      <c r="K359" t="n">
+        <v>0</v>
+      </c>
+      <c r="L359" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Flamengo vs Mirassol</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Flamengo</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E360" t="inlineStr"/>
+      <c r="F360" t="inlineStr"/>
+      <c r="G360" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H360" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I360" t="n">
+        <v>0</v>
+      </c>
+      <c r="J360" t="n">
+        <v>0</v>
+      </c>
+      <c r="K360" t="n">
+        <v>0</v>
+      </c>
+      <c r="L360" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Colegiales vs Midland</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr"/>
+      <c r="F361" t="inlineStr"/>
+      <c r="G361" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H361" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I361" t="n">
+        <v>0</v>
+      </c>
+      <c r="J361" t="n">
+        <v>0</v>
+      </c>
+      <c r="K361" t="n">
+        <v>0</v>
+      </c>
+      <c r="L361" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Charleston Battery vs Hartford Athletic</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Charleston Battery</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E362" t="inlineStr"/>
+      <c r="F362" t="inlineStr"/>
+      <c r="G362" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H362" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I362" t="n">
+        <v>0</v>
+      </c>
+      <c r="J362" t="n">
+        <v>0</v>
+      </c>
+      <c r="K362" t="n">
+        <v>0</v>
+      </c>
+      <c r="L362" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -15621,7 +17165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15732,6 +17276,22 @@
       </c>
       <c r="E6" t="n">
         <v>44</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>34</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-04
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L362"/>
+  <dimension ref="A1:L410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15543,8 +15543,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E329" t="inlineStr"/>
-      <c r="F329" t="inlineStr"/>
       <c r="G329" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -15591,8 +15589,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E330" t="inlineStr"/>
-      <c r="F330" t="inlineStr"/>
       <c r="G330" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -15639,8 +15635,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E331" t="inlineStr"/>
-      <c r="F331" t="inlineStr"/>
       <c r="G331" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -15687,8 +15681,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E332" t="inlineStr"/>
-      <c r="F332" t="inlineStr"/>
       <c r="G332" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -15735,8 +15727,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E333" t="inlineStr"/>
-      <c r="F333" t="inlineStr"/>
       <c r="G333" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -15783,8 +15773,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E334" t="inlineStr"/>
-      <c r="F334" t="inlineStr"/>
       <c r="G334" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -15831,8 +15819,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E335" t="inlineStr"/>
-      <c r="F335" t="inlineStr"/>
       <c r="G335" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -15879,8 +15865,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E336" t="inlineStr"/>
-      <c r="F336" t="inlineStr"/>
       <c r="G336" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -15927,8 +15911,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E337" t="inlineStr"/>
-      <c r="F337" t="inlineStr"/>
       <c r="G337" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -15975,8 +15957,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E338" t="inlineStr"/>
-      <c r="F338" t="inlineStr"/>
       <c r="G338" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16023,8 +16003,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E339" t="inlineStr"/>
-      <c r="F339" t="inlineStr"/>
       <c r="G339" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16071,8 +16049,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E340" t="inlineStr"/>
-      <c r="F340" t="inlineStr"/>
       <c r="G340" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16119,8 +16095,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E341" t="inlineStr"/>
-      <c r="F341" t="inlineStr"/>
       <c r="G341" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16167,8 +16141,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E342" t="inlineStr"/>
-      <c r="F342" t="inlineStr"/>
       <c r="G342" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16215,8 +16187,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E343" t="inlineStr"/>
-      <c r="F343" t="inlineStr"/>
       <c r="G343" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16263,8 +16233,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E344" t="inlineStr"/>
-      <c r="F344" t="inlineStr"/>
       <c r="G344" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16311,8 +16279,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E345" t="inlineStr"/>
-      <c r="F345" t="inlineStr"/>
       <c r="G345" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16359,8 +16325,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E346" t="inlineStr"/>
-      <c r="F346" t="inlineStr"/>
       <c r="G346" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16407,8 +16371,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E347" t="inlineStr"/>
-      <c r="F347" t="inlineStr"/>
       <c r="G347" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16455,8 +16417,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E348" t="inlineStr"/>
-      <c r="F348" t="inlineStr"/>
       <c r="G348" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16503,8 +16463,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E349" t="inlineStr"/>
-      <c r="F349" t="inlineStr"/>
       <c r="G349" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16551,8 +16509,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E350" t="inlineStr"/>
-      <c r="F350" t="inlineStr"/>
       <c r="G350" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16599,8 +16555,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E351" t="inlineStr"/>
-      <c r="F351" t="inlineStr"/>
       <c r="G351" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16647,8 +16601,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E352" t="inlineStr"/>
-      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16695,8 +16647,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E353" t="inlineStr"/>
-      <c r="F353" t="inlineStr"/>
       <c r="G353" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16743,8 +16693,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E354" t="inlineStr"/>
-      <c r="F354" t="inlineStr"/>
       <c r="G354" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16791,8 +16739,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E355" t="inlineStr"/>
-      <c r="F355" t="inlineStr"/>
       <c r="G355" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16839,8 +16785,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E356" t="inlineStr"/>
-      <c r="F356" t="inlineStr"/>
       <c r="G356" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16887,8 +16831,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E357" t="inlineStr"/>
-      <c r="F357" t="inlineStr"/>
       <c r="G357" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16935,8 +16877,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E358" t="inlineStr"/>
-      <c r="F358" t="inlineStr"/>
       <c r="G358" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -16983,8 +16923,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E359" t="inlineStr"/>
-      <c r="F359" t="inlineStr"/>
       <c r="G359" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -17031,8 +16969,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E360" t="inlineStr"/>
-      <c r="F360" t="inlineStr"/>
       <c r="G360" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -17079,8 +17015,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E361" t="inlineStr"/>
-      <c r="F361" t="inlineStr"/>
       <c r="G361" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -17127,8 +17061,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E362" t="inlineStr"/>
-      <c r="F362" t="inlineStr"/>
       <c r="G362" t="inlineStr">
         <is>
           <t>sin resolver</t>
@@ -17149,6 +17081,2310 @@
         <v>0</v>
       </c>
       <c r="L362" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Panthere FC vs Rayon Sport</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Panthere FC</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr"/>
+      <c r="F363" t="inlineStr"/>
+      <c r="G363" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H363" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I363" t="n">
+        <v>0</v>
+      </c>
+      <c r="J363" t="n">
+        <v>0</v>
+      </c>
+      <c r="K363" t="n">
+        <v>0</v>
+      </c>
+      <c r="L363" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Abha vs Al Ettifaq</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Al Ettifaq</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E364" t="inlineStr"/>
+      <c r="F364" t="inlineStr"/>
+      <c r="G364" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H364" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I364" t="n">
+        <v>0</v>
+      </c>
+      <c r="J364" t="n">
+        <v>0</v>
+      </c>
+      <c r="K364" t="n">
+        <v>0</v>
+      </c>
+      <c r="L364" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Arminia Bielefeld vs St. Pauli</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Arminia Bielefeld</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr"/>
+      <c r="F365" t="inlineStr"/>
+      <c r="G365" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H365" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I365" t="n">
+        <v>0</v>
+      </c>
+      <c r="J365" t="n">
+        <v>0</v>
+      </c>
+      <c r="K365" t="n">
+        <v>0</v>
+      </c>
+      <c r="L365" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Hannover 96 vs Karlsruher SC</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Hannover 96</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E366" t="inlineStr"/>
+      <c r="F366" t="inlineStr"/>
+      <c r="G366" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H366" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I366" t="n">
+        <v>0</v>
+      </c>
+      <c r="J366" t="n">
+        <v>0</v>
+      </c>
+      <c r="K366" t="n">
+        <v>0</v>
+      </c>
+      <c r="L366" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Lyon vs AJ Auxerre</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr"/>
+      <c r="F367" t="inlineStr"/>
+      <c r="G367" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H367" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I367" t="n">
+        <v>0</v>
+      </c>
+      <c r="J367" t="n">
+        <v>0</v>
+      </c>
+      <c r="K367" t="n">
+        <v>0</v>
+      </c>
+      <c r="L367" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Viborg FF vs Lyngby Boldklub</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>Viborg FF</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E368" t="inlineStr"/>
+      <c r="F368" t="inlineStr"/>
+      <c r="G368" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H368" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I368" t="n">
+        <v>0</v>
+      </c>
+      <c r="J368" t="n">
+        <v>0</v>
+      </c>
+      <c r="K368" t="n">
+        <v>0</v>
+      </c>
+      <c r="L368" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Aalesund vs IK Start</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>Aalesund</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr"/>
+      <c r="F369" t="inlineStr"/>
+      <c r="G369" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H369" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I369" t="n">
+        <v>0</v>
+      </c>
+      <c r="J369" t="n">
+        <v>0</v>
+      </c>
+      <c r="K369" t="n">
+        <v>0</v>
+      </c>
+      <c r="L369" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Fredrikstad vs Bodo/Glimt</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Bodo/Glimt</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E370" t="inlineStr"/>
+      <c r="F370" t="inlineStr"/>
+      <c r="G370" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H370" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I370" t="n">
+        <v>0</v>
+      </c>
+      <c r="J370" t="n">
+        <v>0</v>
+      </c>
+      <c r="K370" t="n">
+        <v>0</v>
+      </c>
+      <c r="L370" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Istanbul Basaksehir vs Galatasaray</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Galatasaray</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E371" t="inlineStr"/>
+      <c r="F371" t="inlineStr"/>
+      <c r="G371" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H371" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I371" t="n">
+        <v>0</v>
+      </c>
+      <c r="J371" t="n">
+        <v>0</v>
+      </c>
+      <c r="K371" t="n">
+        <v>0</v>
+      </c>
+      <c r="L371" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Marumo Gallants vs Polokwane City FC</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Marumo Gallants</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E372" t="inlineStr"/>
+      <c r="F372" t="inlineStr"/>
+      <c r="G372" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H372" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I372" t="n">
+        <v>0</v>
+      </c>
+      <c r="J372" t="n">
+        <v>0</v>
+      </c>
+      <c r="K372" t="n">
+        <v>0</v>
+      </c>
+      <c r="L372" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Sparta Rotterdam vs PEC Zwolle</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Sparta Rotterdam</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E373" t="inlineStr"/>
+      <c r="F373" t="inlineStr"/>
+      <c r="G373" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H373" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I373" t="n">
+        <v>0</v>
+      </c>
+      <c r="J373" t="n">
+        <v>0</v>
+      </c>
+      <c r="K373" t="n">
+        <v>0</v>
+      </c>
+      <c r="L373" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>JS Saoura vs Horoya</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>JS Saoura</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E374" t="inlineStr"/>
+      <c r="F374" t="inlineStr"/>
+      <c r="G374" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H374" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I374" t="n">
+        <v>0</v>
+      </c>
+      <c r="J374" t="n">
+        <v>0</v>
+      </c>
+      <c r="K374" t="n">
+        <v>0</v>
+      </c>
+      <c r="L374" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Dunkerque vs Clermont Foot</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Dunkerque</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E375" t="inlineStr"/>
+      <c r="F375" t="inlineStr"/>
+      <c r="G375" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H375" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I375" t="n">
+        <v>0</v>
+      </c>
+      <c r="J375" t="n">
+        <v>0</v>
+      </c>
+      <c r="K375" t="n">
+        <v>0</v>
+      </c>
+      <c r="L375" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Grenoble vs Annecy</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Annecy</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E376" t="inlineStr"/>
+      <c r="F376" t="inlineStr"/>
+      <c r="G376" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H376" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I376" t="n">
+        <v>0</v>
+      </c>
+      <c r="J376" t="n">
+        <v>0</v>
+      </c>
+      <c r="K376" t="n">
+        <v>0</v>
+      </c>
+      <c r="L376" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Stade Laval vs Red Star FC 93</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Red Star FC 93</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E377" t="inlineStr"/>
+      <c r="F377" t="inlineStr"/>
+      <c r="G377" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H377" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I377" t="n">
+        <v>0</v>
+      </c>
+      <c r="J377" t="n">
+        <v>0</v>
+      </c>
+      <c r="K377" t="n">
+        <v>0</v>
+      </c>
+      <c r="L377" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Pau vs Sochaux</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Pau</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E378" t="inlineStr"/>
+      <c r="F378" t="inlineStr"/>
+      <c r="G378" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H378" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I378" t="n">
+        <v>0</v>
+      </c>
+      <c r="J378" t="n">
+        <v>0</v>
+      </c>
+      <c r="K378" t="n">
+        <v>0</v>
+      </c>
+      <c r="L378" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Almere City vs Jong Ajax</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Almere City</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E379" t="inlineStr"/>
+      <c r="F379" t="inlineStr"/>
+      <c r="G379" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H379" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I379" t="n">
+        <v>0</v>
+      </c>
+      <c r="J379" t="n">
+        <v>0</v>
+      </c>
+      <c r="K379" t="n">
+        <v>0</v>
+      </c>
+      <c r="L379" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>FC Emmen vs FC Volendam</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>FC Emmen</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E380" t="inlineStr"/>
+      <c r="F380" t="inlineStr"/>
+      <c r="G380" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H380" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I380" t="n">
+        <v>0</v>
+      </c>
+      <c r="J380" t="n">
+        <v>0</v>
+      </c>
+      <c r="K380" t="n">
+        <v>0</v>
+      </c>
+      <c r="L380" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Heracles Almelo vs De Graafschap</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>Heracles Almelo</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E381" t="inlineStr"/>
+      <c r="F381" t="inlineStr"/>
+      <c r="G381" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H381" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I381" t="n">
+        <v>0</v>
+      </c>
+      <c r="J381" t="n">
+        <v>0</v>
+      </c>
+      <c r="K381" t="n">
+        <v>0</v>
+      </c>
+      <c r="L381" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Vitesse vs TOP Oss</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Vitesse</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E382" t="inlineStr"/>
+      <c r="F382" t="inlineStr"/>
+      <c r="G382" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H382" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I382" t="n">
+        <v>0</v>
+      </c>
+      <c r="J382" t="n">
+        <v>0</v>
+      </c>
+      <c r="K382" t="n">
+        <v>0</v>
+      </c>
+      <c r="L382" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>RKC Waalwijk vs NAC Breda</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>NAC Breda</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E383" t="inlineStr"/>
+      <c r="F383" t="inlineStr"/>
+      <c r="G383" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H383" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I383" t="n">
+        <v>0</v>
+      </c>
+      <c r="J383" t="n">
+        <v>0</v>
+      </c>
+      <c r="K383" t="n">
+        <v>0</v>
+      </c>
+      <c r="L383" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>FC Cajamarca vs Cienciano del Cusco</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Cienciano del Cusco</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E384" t="inlineStr"/>
+      <c r="F384" t="inlineStr"/>
+      <c r="G384" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H384" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I384" t="n">
+        <v>0</v>
+      </c>
+      <c r="J384" t="n">
+        <v>0</v>
+      </c>
+      <c r="K384" t="n">
+        <v>0</v>
+      </c>
+      <c r="L384" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Al Ahli vs Al Riyadh</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Al Ahli</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E385" t="inlineStr"/>
+      <c r="F385" t="inlineStr"/>
+      <c r="G385" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H385" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I385" t="n">
+        <v>0</v>
+      </c>
+      <c r="J385" t="n">
+        <v>0</v>
+      </c>
+      <c r="K385" t="n">
+        <v>0</v>
+      </c>
+      <c r="L385" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Al Shabab vs Al Hilal</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Al Hilal</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E386" t="inlineStr"/>
+      <c r="F386" t="inlineStr"/>
+      <c r="G386" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H386" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I386" t="n">
+        <v>0</v>
+      </c>
+      <c r="J386" t="n">
+        <v>0</v>
+      </c>
+      <c r="K386" t="n">
+        <v>0</v>
+      </c>
+      <c r="L386" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart vs FC Cologne</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E387" t="inlineStr"/>
+      <c r="F387" t="inlineStr"/>
+      <c r="G387" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H387" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I387" t="n">
+        <v>0</v>
+      </c>
+      <c r="J387" t="n">
+        <v>0</v>
+      </c>
+      <c r="K387" t="n">
+        <v>0</v>
+      </c>
+      <c r="L387" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Livingston vs Stenhousemuir</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Livingston</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E388" t="inlineStr"/>
+      <c r="F388" t="inlineStr"/>
+      <c r="G388" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H388" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I388" t="n">
+        <v>0</v>
+      </c>
+      <c r="J388" t="n">
+        <v>0</v>
+      </c>
+      <c r="K388" t="n">
+        <v>0</v>
+      </c>
+      <c r="L388" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Defensores de Belgrano vs Racing (Córdoba)</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Defensores de Belgrano</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E389" t="inlineStr"/>
+      <c r="F389" t="inlineStr"/>
+      <c r="G389" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H389" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I389" t="n">
+        <v>0</v>
+      </c>
+      <c r="J389" t="n">
+        <v>0</v>
+      </c>
+      <c r="K389" t="n">
+        <v>0</v>
+      </c>
+      <c r="L389" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Las Palmas vs Leganés</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Las Palmas</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E390" t="inlineStr"/>
+      <c r="F390" t="inlineStr"/>
+      <c r="G390" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H390" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I390" t="n">
+        <v>0</v>
+      </c>
+      <c r="J390" t="n">
+        <v>0</v>
+      </c>
+      <c r="K390" t="n">
+        <v>0</v>
+      </c>
+      <c r="L390" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Genoa vs Como</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E391" t="inlineStr"/>
+      <c r="F391" t="inlineStr"/>
+      <c r="G391" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H391" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I391" t="n">
+        <v>0</v>
+      </c>
+      <c r="J391" t="n">
+        <v>0</v>
+      </c>
+      <c r="K391" t="n">
+        <v>0</v>
+      </c>
+      <c r="L391" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Altrincham vs Eastleigh</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Altrincham</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr"/>
+      <c r="F392" t="inlineStr"/>
+      <c r="G392" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H392" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I392" t="n">
+        <v>0</v>
+      </c>
+      <c r="J392" t="n">
+        <v>0</v>
+      </c>
+      <c r="K392" t="n">
+        <v>0</v>
+      </c>
+      <c r="L392" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Flackwell Heath vs Hanwell Town FC</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Hanwell Town FC</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr"/>
+      <c r="F393" t="inlineStr"/>
+      <c r="G393" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H393" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I393" t="n">
+        <v>0</v>
+      </c>
+      <c r="J393" t="n">
+        <v>0</v>
+      </c>
+      <c r="K393" t="n">
+        <v>0</v>
+      </c>
+      <c r="L393" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Three Bridges vs Kingstonian</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Three Bridges</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E394" t="inlineStr"/>
+      <c r="F394" t="inlineStr"/>
+      <c r="G394" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H394" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I394" t="n">
+        <v>0</v>
+      </c>
+      <c r="J394" t="n">
+        <v>0</v>
+      </c>
+      <c r="K394" t="n">
+        <v>0</v>
+      </c>
+      <c r="L394" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Ipswich Town vs Liverpool</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Liverpool</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E395" t="inlineStr"/>
+      <c r="F395" t="inlineStr"/>
+      <c r="G395" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H395" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I395" t="n">
+        <v>0</v>
+      </c>
+      <c r="J395" t="n">
+        <v>0</v>
+      </c>
+      <c r="K395" t="n">
+        <v>0</v>
+      </c>
+      <c r="L395" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Real Betis vs Real Madrid</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E396" t="inlineStr"/>
+      <c r="F396" t="inlineStr"/>
+      <c r="G396" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H396" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I396" t="n">
+        <v>0</v>
+      </c>
+      <c r="J396" t="n">
+        <v>0</v>
+      </c>
+      <c r="K396" t="n">
+        <v>0</v>
+      </c>
+      <c r="L396" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Sandefjord vs Viking FK</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Viking FK</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr"/>
+      <c r="F397" t="inlineStr"/>
+      <c r="G397" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H397" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I397" t="n">
+        <v>0</v>
+      </c>
+      <c r="J397" t="n">
+        <v>0</v>
+      </c>
+      <c r="K397" t="n">
+        <v>0</v>
+      </c>
+      <c r="L397" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Real Oruro vs San Antonio Bulo Bulo</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Real Oruro</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E398" t="inlineStr"/>
+      <c r="F398" t="inlineStr"/>
+      <c r="G398" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H398" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I398" t="n">
+        <v>0</v>
+      </c>
+      <c r="J398" t="n">
+        <v>0</v>
+      </c>
+      <c r="K398" t="n">
+        <v>0</v>
+      </c>
+      <c r="L398" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain vs AS Monaco</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E399" t="inlineStr"/>
+      <c r="F399" t="inlineStr"/>
+      <c r="G399" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H399" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I399" t="n">
+        <v>0</v>
+      </c>
+      <c r="J399" t="n">
+        <v>0</v>
+      </c>
+      <c r="K399" t="n">
+        <v>0</v>
+      </c>
+      <c r="L399" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>FC Porto vs Moreirense</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>FC Porto</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr"/>
+      <c r="F400" t="inlineStr"/>
+      <c r="G400" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H400" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I400" t="n">
+        <v>0</v>
+      </c>
+      <c r="J400" t="n">
+        <v>0</v>
+      </c>
+      <c r="K400" t="n">
+        <v>0</v>
+      </c>
+      <c r="L400" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Alianza Atlético vs UTC</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Alianza Atlético</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr"/>
+      <c r="F401" t="inlineStr"/>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I401" t="n">
+        <v>0</v>
+      </c>
+      <c r="J401" t="n">
+        <v>0</v>
+      </c>
+      <c r="K401" t="n">
+        <v>0</v>
+      </c>
+      <c r="L401" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>ABB vs Universitario de Vinto</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>ABB</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr"/>
+      <c r="F402" t="inlineStr"/>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I402" t="n">
+        <v>0</v>
+      </c>
+      <c r="J402" t="n">
+        <v>0</v>
+      </c>
+      <c r="K402" t="n">
+        <v>0</v>
+      </c>
+      <c r="L402" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Belgrano (Córdoba) vs Huracán</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Belgrano (Córdoba)</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr"/>
+      <c r="F403" t="inlineStr"/>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I403" t="n">
+        <v>0</v>
+      </c>
+      <c r="J403" t="n">
+        <v>0</v>
+      </c>
+      <c r="K403" t="n">
+        <v>0</v>
+      </c>
+      <c r="L403" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Platense vs Deportivo Riestra</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Platense</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr"/>
+      <c r="F404" t="inlineStr"/>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I404" t="n">
+        <v>0</v>
+      </c>
+      <c r="J404" t="n">
+        <v>0</v>
+      </c>
+      <c r="K404" t="n">
+        <v>0</v>
+      </c>
+      <c r="L404" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Criciúma vs Cuiabá</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Criciúma</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr"/>
+      <c r="F405" t="inlineStr"/>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I405" t="n">
+        <v>0</v>
+      </c>
+      <c r="J405" t="n">
+        <v>0</v>
+      </c>
+      <c r="K405" t="n">
+        <v>0</v>
+      </c>
+      <c r="L405" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Loudoun United FC vs Colorado Springs Switchbacks FC</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Colorado Springs Switchbacks FC</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr"/>
+      <c r="F406" t="inlineStr"/>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I406" t="n">
+        <v>0</v>
+      </c>
+      <c r="J406" t="n">
+        <v>0</v>
+      </c>
+      <c r="K406" t="n">
+        <v>0</v>
+      </c>
+      <c r="L406" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>CRB vs América Mineiro</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>CRB</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr"/>
+      <c r="F407" t="inlineStr"/>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I407" t="n">
+        <v>0</v>
+      </c>
+      <c r="J407" t="n">
+        <v>0</v>
+      </c>
+      <c r="K407" t="n">
+        <v>0</v>
+      </c>
+      <c r="L407" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Deportes Concepcion vs Audax Italiano</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Deportes Concepcion</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr"/>
+      <c r="F408" t="inlineStr"/>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I408" t="n">
+        <v>0</v>
+      </c>
+      <c r="J408" t="n">
+        <v>0</v>
+      </c>
+      <c r="K408" t="n">
+        <v>0</v>
+      </c>
+      <c r="L408" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Antigua GFC vs Aurora FC</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Antigua GFC</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr"/>
+      <c r="F409" t="inlineStr"/>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I409" t="n">
+        <v>0</v>
+      </c>
+      <c r="J409" t="n">
+        <v>0</v>
+      </c>
+      <c r="K409" t="n">
+        <v>0</v>
+      </c>
+      <c r="L409" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>FC Juarez vs Pachuca</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>FC Juarez</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr"/>
+      <c r="F410" t="inlineStr"/>
+      <c r="G410" t="inlineStr">
+        <is>
+          <t>sin resolver</t>
+        </is>
+      </c>
+      <c r="H410" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="I410" t="n">
+        <v>0</v>
+      </c>
+      <c r="J410" t="n">
+        <v>0</v>
+      </c>
+      <c r="K410" t="n">
+        <v>0</v>
+      </c>
+      <c r="L410" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -17165,7 +19401,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17292,6 +19528,22 @@
       </c>
       <c r="E7" t="n">
         <v>96</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>48</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-08
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L670"/>
+  <dimension ref="A1:L704"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26307,8 +26307,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E563" t="inlineStr"/>
-      <c r="F563" t="inlineStr"/>
       <c r="G563" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -26355,8 +26353,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E564" t="inlineStr"/>
-      <c r="F564" t="inlineStr"/>
       <c r="G564" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -26403,8 +26399,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E565" t="inlineStr"/>
-      <c r="F565" t="inlineStr"/>
       <c r="G565" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -26451,8 +26445,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E566" t="inlineStr"/>
-      <c r="F566" t="inlineStr"/>
       <c r="G566" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -26499,8 +26491,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E567" t="inlineStr"/>
-      <c r="F567" t="inlineStr"/>
       <c r="G567" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -26547,8 +26537,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E568" t="inlineStr"/>
-      <c r="F568" t="inlineStr"/>
       <c r="G568" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -26595,8 +26583,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E569" t="inlineStr"/>
-      <c r="F569" t="inlineStr"/>
       <c r="G569" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -26643,8 +26629,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E570" t="inlineStr"/>
-      <c r="F570" t="inlineStr"/>
       <c r="G570" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -26691,8 +26675,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E571" t="inlineStr"/>
-      <c r="F571" t="inlineStr"/>
       <c r="G571" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -26739,8 +26721,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E572" t="inlineStr"/>
-      <c r="F572" t="inlineStr"/>
       <c r="G572" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -26787,8 +26767,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E573" t="inlineStr"/>
-      <c r="F573" t="inlineStr"/>
       <c r="G573" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -26835,8 +26813,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E574" t="inlineStr"/>
-      <c r="F574" t="inlineStr"/>
       <c r="G574" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -26883,8 +26859,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E575" t="inlineStr"/>
-      <c r="F575" t="inlineStr"/>
       <c r="G575" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -26931,8 +26905,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E576" t="inlineStr"/>
-      <c r="F576" t="inlineStr"/>
       <c r="G576" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -26979,8 +26951,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E577" t="inlineStr"/>
-      <c r="F577" t="inlineStr"/>
       <c r="G577" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -27027,8 +26997,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E578" t="inlineStr"/>
-      <c r="F578" t="inlineStr"/>
       <c r="G578" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -27075,8 +27043,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E579" t="inlineStr"/>
-      <c r="F579" t="inlineStr"/>
       <c r="G579" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -27123,8 +27089,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E580" t="inlineStr"/>
-      <c r="F580" t="inlineStr"/>
       <c r="G580" t="inlineStr">
         <is>
           <t>2-5</t>
@@ -27171,8 +27135,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E581" t="inlineStr"/>
-      <c r="F581" t="inlineStr"/>
       <c r="G581" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -27219,8 +27181,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E582" t="inlineStr"/>
-      <c r="F582" t="inlineStr"/>
       <c r="G582" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -27267,8 +27227,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E583" t="inlineStr"/>
-      <c r="F583" t="inlineStr"/>
       <c r="G583" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -27315,8 +27273,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E584" t="inlineStr"/>
-      <c r="F584" t="inlineStr"/>
       <c r="G584" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -27363,8 +27319,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E585" t="inlineStr"/>
-      <c r="F585" t="inlineStr"/>
       <c r="G585" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -27411,8 +27365,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E586" t="inlineStr"/>
-      <c r="F586" t="inlineStr"/>
       <c r="G586" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -27459,8 +27411,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E587" t="inlineStr"/>
-      <c r="F587" t="inlineStr"/>
       <c r="G587" t="inlineStr">
         <is>
           <t>2-6</t>
@@ -27507,8 +27457,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E588" t="inlineStr"/>
-      <c r="F588" t="inlineStr"/>
       <c r="G588" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -27555,8 +27503,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E589" t="inlineStr"/>
-      <c r="F589" t="inlineStr"/>
       <c r="G589" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -27603,8 +27549,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E590" t="inlineStr"/>
-      <c r="F590" t="inlineStr"/>
       <c r="G590" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -27651,8 +27595,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E591" t="inlineStr"/>
-      <c r="F591" t="inlineStr"/>
       <c r="G591" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -27699,8 +27641,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E592" t="inlineStr"/>
-      <c r="F592" t="inlineStr"/>
       <c r="G592" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -27747,8 +27687,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E593" t="inlineStr"/>
-      <c r="F593" t="inlineStr"/>
       <c r="G593" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -27795,8 +27733,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E594" t="inlineStr"/>
-      <c r="F594" t="inlineStr"/>
       <c r="G594" t="inlineStr">
         <is>
           <t>0-5</t>
@@ -27843,8 +27779,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E595" t="inlineStr"/>
-      <c r="F595" t="inlineStr"/>
       <c r="G595" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -27891,8 +27825,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E596" t="inlineStr"/>
-      <c r="F596" t="inlineStr"/>
       <c r="G596" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -27939,8 +27871,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E597" t="inlineStr"/>
-      <c r="F597" t="inlineStr"/>
       <c r="G597" t="inlineStr">
         <is>
           <t>0-5</t>
@@ -27987,8 +27917,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E598" t="inlineStr"/>
-      <c r="F598" t="inlineStr"/>
       <c r="G598" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -28035,8 +27963,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E599" t="inlineStr"/>
-      <c r="F599" t="inlineStr"/>
       <c r="G599" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -28083,8 +28009,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E600" t="inlineStr"/>
-      <c r="F600" t="inlineStr"/>
       <c r="G600" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -28131,8 +28055,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E601" t="inlineStr"/>
-      <c r="F601" t="inlineStr"/>
       <c r="G601" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -28179,8 +28101,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E602" t="inlineStr"/>
-      <c r="F602" t="inlineStr"/>
       <c r="G602" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -28227,8 +28147,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E603" t="inlineStr"/>
-      <c r="F603" t="inlineStr"/>
       <c r="G603" t="inlineStr">
         <is>
           <t>0-5</t>
@@ -28275,8 +28193,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E604" t="inlineStr"/>
-      <c r="F604" t="inlineStr"/>
       <c r="G604" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -28323,8 +28239,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E605" t="inlineStr"/>
-      <c r="F605" t="inlineStr"/>
       <c r="G605" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -28371,8 +28285,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E606" t="inlineStr"/>
-      <c r="F606" t="inlineStr"/>
       <c r="G606" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -28419,8 +28331,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E607" t="inlineStr"/>
-      <c r="F607" t="inlineStr"/>
       <c r="G607" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -28467,8 +28377,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E608" t="inlineStr"/>
-      <c r="F608" t="inlineStr"/>
       <c r="G608" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -28515,8 +28423,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E609" t="inlineStr"/>
-      <c r="F609" t="inlineStr"/>
       <c r="G609" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -28563,8 +28469,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E610" t="inlineStr"/>
-      <c r="F610" t="inlineStr"/>
       <c r="G610" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -28611,8 +28515,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E611" t="inlineStr"/>
-      <c r="F611" t="inlineStr"/>
       <c r="G611" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -28659,8 +28561,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E612" t="inlineStr"/>
-      <c r="F612" t="inlineStr"/>
       <c r="G612" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -28707,8 +28607,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E613" t="inlineStr"/>
-      <c r="F613" t="inlineStr"/>
       <c r="G613" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -28755,8 +28653,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E614" t="inlineStr"/>
-      <c r="F614" t="inlineStr"/>
       <c r="G614" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -28803,8 +28699,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E615" t="inlineStr"/>
-      <c r="F615" t="inlineStr"/>
       <c r="G615" t="inlineStr">
         <is>
           <t>1-4</t>
@@ -28851,8 +28745,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E616" t="inlineStr"/>
-      <c r="F616" t="inlineStr"/>
       <c r="G616" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -28899,8 +28791,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E617" t="inlineStr"/>
-      <c r="F617" t="inlineStr"/>
       <c r="G617" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -28947,8 +28837,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E618" t="inlineStr"/>
-      <c r="F618" t="inlineStr"/>
       <c r="G618" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -28995,8 +28883,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E619" t="inlineStr"/>
-      <c r="F619" t="inlineStr"/>
       <c r="G619" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -29043,8 +28929,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E620" t="inlineStr"/>
-      <c r="F620" t="inlineStr"/>
       <c r="G620" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -29091,8 +28975,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E621" t="inlineStr"/>
-      <c r="F621" t="inlineStr"/>
       <c r="G621" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -29139,8 +29021,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E622" t="inlineStr"/>
-      <c r="F622" t="inlineStr"/>
       <c r="G622" t="inlineStr">
         <is>
           <t>5-2</t>
@@ -29187,8 +29067,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E623" t="inlineStr"/>
-      <c r="F623" t="inlineStr"/>
       <c r="G623" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -29235,8 +29113,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E624" t="inlineStr"/>
-      <c r="F624" t="inlineStr"/>
       <c r="G624" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -29283,8 +29159,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E625" t="inlineStr"/>
-      <c r="F625" t="inlineStr"/>
       <c r="G625" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -29331,8 +29205,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E626" t="inlineStr"/>
-      <c r="F626" t="inlineStr"/>
       <c r="G626" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -29379,8 +29251,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E627" t="inlineStr"/>
-      <c r="F627" t="inlineStr"/>
       <c r="G627" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -29427,8 +29297,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E628" t="inlineStr"/>
-      <c r="F628" t="inlineStr"/>
       <c r="G628" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -29475,8 +29343,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E629" t="inlineStr"/>
-      <c r="F629" t="inlineStr"/>
       <c r="G629" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -29523,8 +29389,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E630" t="inlineStr"/>
-      <c r="F630" t="inlineStr"/>
       <c r="G630" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -29571,8 +29435,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E631" t="inlineStr"/>
-      <c r="F631" t="inlineStr"/>
       <c r="G631" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -29619,8 +29481,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E632" t="inlineStr"/>
-      <c r="F632" t="inlineStr"/>
       <c r="G632" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -29667,8 +29527,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E633" t="inlineStr"/>
-      <c r="F633" t="inlineStr"/>
       <c r="G633" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -29715,8 +29573,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E634" t="inlineStr"/>
-      <c r="F634" t="inlineStr"/>
       <c r="G634" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -29763,8 +29619,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E635" t="inlineStr"/>
-      <c r="F635" t="inlineStr"/>
       <c r="G635" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -29811,8 +29665,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E636" t="inlineStr"/>
-      <c r="F636" t="inlineStr"/>
       <c r="G636" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -29859,8 +29711,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E637" t="inlineStr"/>
-      <c r="F637" t="inlineStr"/>
       <c r="G637" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -29907,8 +29757,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E638" t="inlineStr"/>
-      <c r="F638" t="inlineStr"/>
       <c r="G638" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -29955,8 +29803,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E639" t="inlineStr"/>
-      <c r="F639" t="inlineStr"/>
       <c r="G639" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -30003,8 +29849,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E640" t="inlineStr"/>
-      <c r="F640" t="inlineStr"/>
       <c r="G640" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -30051,8 +29895,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E641" t="inlineStr"/>
-      <c r="F641" t="inlineStr"/>
       <c r="G641" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -30099,8 +29941,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E642" t="inlineStr"/>
-      <c r="F642" t="inlineStr"/>
       <c r="G642" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -30147,8 +29987,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E643" t="inlineStr"/>
-      <c r="F643" t="inlineStr"/>
       <c r="G643" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -30195,8 +30033,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E644" t="inlineStr"/>
-      <c r="F644" t="inlineStr"/>
       <c r="G644" t="inlineStr">
         <is>
           <t>4-2</t>
@@ -30243,8 +30079,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E645" t="inlineStr"/>
-      <c r="F645" t="inlineStr"/>
       <c r="G645" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -30291,8 +30125,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E646" t="inlineStr"/>
-      <c r="F646" t="inlineStr"/>
       <c r="G646" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -30339,8 +30171,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E647" t="inlineStr"/>
-      <c r="F647" t="inlineStr"/>
       <c r="G647" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -30387,8 +30217,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E648" t="inlineStr"/>
-      <c r="F648" t="inlineStr"/>
       <c r="G648" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -30435,8 +30263,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E649" t="inlineStr"/>
-      <c r="F649" t="inlineStr"/>
       <c r="G649" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -30483,8 +30309,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E650" t="inlineStr"/>
-      <c r="F650" t="inlineStr"/>
       <c r="G650" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -30531,8 +30355,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E651" t="inlineStr"/>
-      <c r="F651" t="inlineStr"/>
       <c r="G651" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -30579,8 +30401,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E652" t="inlineStr"/>
-      <c r="F652" t="inlineStr"/>
       <c r="G652" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -30627,8 +30447,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E653" t="inlineStr"/>
-      <c r="F653" t="inlineStr"/>
       <c r="G653" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -30675,8 +30493,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E654" t="inlineStr"/>
-      <c r="F654" t="inlineStr"/>
       <c r="G654" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -30723,8 +30539,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E655" t="inlineStr"/>
-      <c r="F655" t="inlineStr"/>
       <c r="G655" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -30771,8 +30585,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E656" t="inlineStr"/>
-      <c r="F656" t="inlineStr"/>
       <c r="G656" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -30819,8 +30631,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E657" t="inlineStr"/>
-      <c r="F657" t="inlineStr"/>
       <c r="G657" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -30867,8 +30677,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E658" t="inlineStr"/>
-      <c r="F658" t="inlineStr"/>
       <c r="G658" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -30915,8 +30723,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E659" t="inlineStr"/>
-      <c r="F659" t="inlineStr"/>
       <c r="G659" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -30963,8 +30769,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E660" t="inlineStr"/>
-      <c r="F660" t="inlineStr"/>
       <c r="G660" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -31011,8 +30815,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E661" t="inlineStr"/>
-      <c r="F661" t="inlineStr"/>
       <c r="G661" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -31059,8 +30861,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E662" t="inlineStr"/>
-      <c r="F662" t="inlineStr"/>
       <c r="G662" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -31107,8 +30907,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E663" t="inlineStr"/>
-      <c r="F663" t="inlineStr"/>
       <c r="G663" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -31155,8 +30953,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E664" t="inlineStr"/>
-      <c r="F664" t="inlineStr"/>
       <c r="G664" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -31203,8 +30999,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E665" t="inlineStr"/>
-      <c r="F665" t="inlineStr"/>
       <c r="G665" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -31251,8 +31045,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E666" t="inlineStr"/>
-      <c r="F666" t="inlineStr"/>
       <c r="G666" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -31299,8 +31091,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E667" t="inlineStr"/>
-      <c r="F667" t="inlineStr"/>
       <c r="G667" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -31347,8 +31137,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E668" t="inlineStr"/>
-      <c r="F668" t="inlineStr"/>
       <c r="G668" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -31395,8 +31183,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E669" t="inlineStr"/>
-      <c r="F669" t="inlineStr"/>
       <c r="G669" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -31443,8 +31229,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E670" t="inlineStr"/>
-      <c r="F670" t="inlineStr"/>
       <c r="G670" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -31465,6 +31249,1638 @@
         <v>0</v>
       </c>
       <c r="L670" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Asteras Tripoli vs Iraklis</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Asteras Tripoli</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr"/>
+      <c r="F671" t="inlineStr"/>
+      <c r="G671" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H671" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I671" t="n">
+        <v>0</v>
+      </c>
+      <c r="J671" t="n">
+        <v>0</v>
+      </c>
+      <c r="K671" t="n">
+        <v>0</v>
+      </c>
+      <c r="L671" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Al Khaleej vs Al Riyadh</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Al Khaleej</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr"/>
+      <c r="F672" t="inlineStr"/>
+      <c r="G672" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H672" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I672" t="n">
+        <v>0</v>
+      </c>
+      <c r="J672" t="n">
+        <v>0</v>
+      </c>
+      <c r="K672" t="n">
+        <v>0</v>
+      </c>
+      <c r="L672" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Cagliari vs Lecce</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Cagliari</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr"/>
+      <c r="F673" t="inlineStr"/>
+      <c r="G673" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H673" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I673" t="n">
+        <v>0</v>
+      </c>
+      <c r="J673" t="n">
+        <v>0</v>
+      </c>
+      <c r="K673" t="n">
+        <v>0</v>
+      </c>
+      <c r="L673" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>FC Midtjylland vs FC Nordsjælland</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>FC Midtjylland</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr"/>
+      <c r="F674" t="inlineStr"/>
+      <c r="G674" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H674" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I674" t="n">
+        <v>0</v>
+      </c>
+      <c r="J674" t="n">
+        <v>0</v>
+      </c>
+      <c r="K674" t="n">
+        <v>0</v>
+      </c>
+      <c r="L674" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Kalmar FF vs Djurgården</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Djurgården</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr"/>
+      <c r="F675" t="inlineStr"/>
+      <c r="G675" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H675" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I675" t="n">
+        <v>0</v>
+      </c>
+      <c r="J675" t="n">
+        <v>0</v>
+      </c>
+      <c r="K675" t="n">
+        <v>0</v>
+      </c>
+      <c r="L675" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Malmö FF vs AIK</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>Malmö FF</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr"/>
+      <c r="F676" t="inlineStr"/>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I676" t="n">
+        <v>0</v>
+      </c>
+      <c r="J676" t="n">
+        <v>0</v>
+      </c>
+      <c r="K676" t="n">
+        <v>0</v>
+      </c>
+      <c r="L676" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Mjällby AIF vs IFK Göteborg</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Mjällby AIF</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr"/>
+      <c r="F677" t="inlineStr"/>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I677" t="n">
+        <v>0</v>
+      </c>
+      <c r="J677" t="n">
+        <v>0</v>
+      </c>
+      <c r="K677" t="n">
+        <v>0</v>
+      </c>
+      <c r="L677" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Goztepe vs Gaziantep FK</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Goztepe</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr"/>
+      <c r="F678" t="inlineStr"/>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I678" t="n">
+        <v>0</v>
+      </c>
+      <c r="J678" t="n">
+        <v>0</v>
+      </c>
+      <c r="K678" t="n">
+        <v>0</v>
+      </c>
+      <c r="L678" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Caykur Rizespor vs Alanyaspor</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Caykur Rizespor</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr"/>
+      <c r="F679" t="inlineStr"/>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I679" t="n">
+        <v>0</v>
+      </c>
+      <c r="J679" t="n">
+        <v>0</v>
+      </c>
+      <c r="K679" t="n">
+        <v>0</v>
+      </c>
+      <c r="L679" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Albion FC vs Progreso</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Albion FC</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr"/>
+      <c r="F680" t="inlineStr"/>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I680" t="n">
+        <v>0</v>
+      </c>
+      <c r="J680" t="n">
+        <v>0</v>
+      </c>
+      <c r="K680" t="n">
+        <v>0</v>
+      </c>
+      <c r="L680" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Jong PSV vs FC Den Bosch</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Jong PSV</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr"/>
+      <c r="F681" t="inlineStr"/>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I681" t="n">
+        <v>0</v>
+      </c>
+      <c r="J681" t="n">
+        <v>0</v>
+      </c>
+      <c r="K681" t="n">
+        <v>0</v>
+      </c>
+      <c r="L681" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Al Hilal vs Neom SC</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>Al Hilal</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr"/>
+      <c r="F682" t="inlineStr"/>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I682" t="n">
+        <v>0</v>
+      </c>
+      <c r="J682" t="n">
+        <v>0</v>
+      </c>
+      <c r="K682" t="n">
+        <v>0</v>
+      </c>
+      <c r="L682" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Jong FC Utrecht vs FC Eindhoven</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Jong FC Utrecht</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr"/>
+      <c r="F683" t="inlineStr"/>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I683" t="n">
+        <v>0</v>
+      </c>
+      <c r="J683" t="n">
+        <v>0</v>
+      </c>
+      <c r="K683" t="n">
+        <v>0</v>
+      </c>
+      <c r="L683" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Palermo vs Sampdoria</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr"/>
+      <c r="F684" t="inlineStr"/>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I684" t="n">
+        <v>0</v>
+      </c>
+      <c r="J684" t="n">
+        <v>0</v>
+      </c>
+      <c r="K684" t="n">
+        <v>0</v>
+      </c>
+      <c r="L684" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>CD Sabadell vs Córdoba</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>CD Sabadell</t>
+        </is>
+      </c>
+      <c r="D685" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E685" t="inlineStr"/>
+      <c r="F685" t="inlineStr"/>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I685" t="n">
+        <v>0</v>
+      </c>
+      <c r="J685" t="n">
+        <v>0</v>
+      </c>
+      <c r="K685" t="n">
+        <v>0</v>
+      </c>
+      <c r="L685" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Nantes vs AS Nancy Lorraine</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="D686" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E686" t="inlineStr"/>
+      <c r="F686" t="inlineStr"/>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I686" t="n">
+        <v>0</v>
+      </c>
+      <c r="J686" t="n">
+        <v>0</v>
+      </c>
+      <c r="K686" t="n">
+        <v>0</v>
+      </c>
+      <c r="L686" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Carshalton Athletic vs Chertsey Town</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Carshalton Athletic</t>
+        </is>
+      </c>
+      <c r="D687" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E687" t="inlineStr"/>
+      <c r="F687" t="inlineStr"/>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I687" t="n">
+        <v>0</v>
+      </c>
+      <c r="J687" t="n">
+        <v>0</v>
+      </c>
+      <c r="K687" t="n">
+        <v>0</v>
+      </c>
+      <c r="L687" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Redditch United vs Malvern Town</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Redditch United</t>
+        </is>
+      </c>
+      <c r="D688" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E688" t="inlineStr"/>
+      <c r="F688" t="inlineStr"/>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I688" t="n">
+        <v>0</v>
+      </c>
+      <c r="J688" t="n">
+        <v>0</v>
+      </c>
+      <c r="K688" t="n">
+        <v>0</v>
+      </c>
+      <c r="L688" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Swindon Supermarine vs Winslow United</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Swindon Supermarine</t>
+        </is>
+      </c>
+      <c r="D689" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E689" t="inlineStr"/>
+      <c r="F689" t="inlineStr"/>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I689" t="n">
+        <v>0</v>
+      </c>
+      <c r="J689" t="n">
+        <v>0</v>
+      </c>
+      <c r="K689" t="n">
+        <v>0</v>
+      </c>
+      <c r="L689" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Bromley vs AFC Wimbledon</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>Bromley</t>
+        </is>
+      </c>
+      <c r="D690" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E690" t="inlineStr"/>
+      <c r="F690" t="inlineStr"/>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I690" t="n">
+        <v>0</v>
+      </c>
+      <c r="J690" t="n">
+        <v>0</v>
+      </c>
+      <c r="K690" t="n">
+        <v>0</v>
+      </c>
+      <c r="L690" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Guaraní vs Deportivo Recoleta</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>Guaraní</t>
+        </is>
+      </c>
+      <c r="D691" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E691" t="inlineStr"/>
+      <c r="F691" t="inlineStr"/>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I691" t="n">
+        <v>0</v>
+      </c>
+      <c r="J691" t="n">
+        <v>0</v>
+      </c>
+      <c r="K691" t="n">
+        <v>0</v>
+      </c>
+      <c r="L691" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Estoril vs Arouca</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Estoril</t>
+        </is>
+      </c>
+      <c r="D692" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E692" t="inlineStr"/>
+      <c r="F692" t="inlineStr"/>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I692" t="n">
+        <v>0</v>
+      </c>
+      <c r="J692" t="n">
+        <v>0</v>
+      </c>
+      <c r="K692" t="n">
+        <v>0</v>
+      </c>
+      <c r="L692" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Elche vs Real Sociedad</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Real Sociedad</t>
+        </is>
+      </c>
+      <c r="D693" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E693" t="inlineStr"/>
+      <c r="F693" t="inlineStr"/>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I693" t="n">
+        <v>0</v>
+      </c>
+      <c r="J693" t="n">
+        <v>0</v>
+      </c>
+      <c r="K693" t="n">
+        <v>0</v>
+      </c>
+      <c r="L693" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Cerro Porteño vs Nacional Asunción</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>Cerro Porteño</t>
+        </is>
+      </c>
+      <c r="D694" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E694" t="inlineStr"/>
+      <c r="F694" t="inlineStr"/>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I694" t="n">
+        <v>0</v>
+      </c>
+      <c r="J694" t="n">
+        <v>0</v>
+      </c>
+      <c r="K694" t="n">
+        <v>0</v>
+      </c>
+      <c r="L694" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Barracas Central vs Argentinos Juniors</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Argentinos Juniors</t>
+        </is>
+      </c>
+      <c r="D695" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E695" t="inlineStr"/>
+      <c r="F695" t="inlineStr"/>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I695" t="n">
+        <v>0</v>
+      </c>
+      <c r="J695" t="n">
+        <v>0</v>
+      </c>
+      <c r="K695" t="n">
+        <v>0</v>
+      </c>
+      <c r="L695" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Carabobo vs Estudiantes de Mérida</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Carabobo</t>
+        </is>
+      </c>
+      <c r="D696" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E696" t="inlineStr"/>
+      <c r="F696" t="inlineStr"/>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I696" t="n">
+        <v>0</v>
+      </c>
+      <c r="J696" t="n">
+        <v>0</v>
+      </c>
+      <c r="K696" t="n">
+        <v>0</v>
+      </c>
+      <c r="L696" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Vitória vs Grêmio</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="D697" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E697" t="inlineStr"/>
+      <c r="F697" t="inlineStr"/>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I697" t="n">
+        <v>0</v>
+      </c>
+      <c r="J697" t="n">
+        <v>0</v>
+      </c>
+      <c r="K697" t="n">
+        <v>0</v>
+      </c>
+      <c r="L697" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>UCV FC vs Academia Puerto Cabello</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Academia Puerto Cabello</t>
+        </is>
+      </c>
+      <c r="D698" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E698" t="inlineStr"/>
+      <c r="F698" t="inlineStr"/>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I698" t="n">
+        <v>0</v>
+      </c>
+      <c r="J698" t="n">
+        <v>0</v>
+      </c>
+      <c r="K698" t="n">
+        <v>0</v>
+      </c>
+      <c r="L698" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Excursionistas vs Ituzaingó</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Excursionistas</t>
+        </is>
+      </c>
+      <c r="D699" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E699" t="inlineStr"/>
+      <c r="F699" t="inlineStr"/>
+      <c r="G699" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H699" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I699" t="n">
+        <v>0</v>
+      </c>
+      <c r="J699" t="n">
+        <v>0</v>
+      </c>
+      <c r="K699" t="n">
+        <v>0</v>
+      </c>
+      <c r="L699" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Deportes Limache vs Cobresal</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Deportes Limache</t>
+        </is>
+      </c>
+      <c r="D700" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E700" t="inlineStr"/>
+      <c r="F700" t="inlineStr"/>
+      <c r="G700" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H700" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I700" t="n">
+        <v>0</v>
+      </c>
+      <c r="J700" t="n">
+        <v>0</v>
+      </c>
+      <c r="K700" t="n">
+        <v>0</v>
+      </c>
+      <c r="L700" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Emelec vs Manta F.C.</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Emelec</t>
+        </is>
+      </c>
+      <c r="D701" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E701" t="inlineStr"/>
+      <c r="F701" t="inlineStr"/>
+      <c r="G701" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I701" t="n">
+        <v>0</v>
+      </c>
+      <c r="J701" t="n">
+        <v>0</v>
+      </c>
+      <c r="K701" t="n">
+        <v>0</v>
+      </c>
+      <c r="L701" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Mushuc Runa vs Leones</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Mushuc Runa</t>
+        </is>
+      </c>
+      <c r="D702" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E702" t="inlineStr"/>
+      <c r="F702" t="inlineStr"/>
+      <c r="G702" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H702" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I702" t="n">
+        <v>0</v>
+      </c>
+      <c r="J702" t="n">
+        <v>0</v>
+      </c>
+      <c r="K702" t="n">
+        <v>0</v>
+      </c>
+      <c r="L702" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Orense vs Guayaquil City FC</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Orense</t>
+        </is>
+      </c>
+      <c r="D703" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E703" t="inlineStr"/>
+      <c r="F703" t="inlineStr"/>
+      <c r="G703" t="inlineStr">
+        <is>
+          <t>4-3</t>
+        </is>
+      </c>
+      <c r="H703" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I703" t="n">
+        <v>0</v>
+      </c>
+      <c r="J703" t="n">
+        <v>0</v>
+      </c>
+      <c r="K703" t="n">
+        <v>0</v>
+      </c>
+      <c r="L703" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Atlético Nacional vs Deportivo Cali</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Atlético Nacional</t>
+        </is>
+      </c>
+      <c r="D704" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E704" t="inlineStr"/>
+      <c r="F704" t="inlineStr"/>
+      <c r="G704" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H704" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I704" t="n">
+        <v>0</v>
+      </c>
+      <c r="J704" t="n">
+        <v>0</v>
+      </c>
+      <c r="K704" t="n">
+        <v>0</v>
+      </c>
+      <c r="L704" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -31481,7 +32897,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31662,6 +33078,25 @@
       </c>
       <c r="E10" t="n">
         <v>108</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>34</v>
+      </c>
+      <c r="C11" t="n">
+        <v>26</v>
+      </c>
+      <c r="D11" t="n">
+        <v>76.5</v>
+      </c>
+      <c r="E11" t="n">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-09
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L704"/>
+  <dimension ref="A1:L748"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -31275,8 +31275,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E671" t="inlineStr"/>
-      <c r="F671" t="inlineStr"/>
       <c r="G671" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -31323,8 +31321,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E672" t="inlineStr"/>
-      <c r="F672" t="inlineStr"/>
       <c r="G672" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -31371,8 +31367,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E673" t="inlineStr"/>
-      <c r="F673" t="inlineStr"/>
       <c r="G673" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -31419,8 +31413,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E674" t="inlineStr"/>
-      <c r="F674" t="inlineStr"/>
       <c r="G674" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -31467,8 +31459,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E675" t="inlineStr"/>
-      <c r="F675" t="inlineStr"/>
       <c r="G675" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -31515,8 +31505,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E676" t="inlineStr"/>
-      <c r="F676" t="inlineStr"/>
       <c r="G676" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -31563,8 +31551,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E677" t="inlineStr"/>
-      <c r="F677" t="inlineStr"/>
       <c r="G677" t="inlineStr">
         <is>
           <t>1-4</t>
@@ -31611,8 +31597,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E678" t="inlineStr"/>
-      <c r="F678" t="inlineStr"/>
       <c r="G678" t="inlineStr">
         <is>
           <t>2-4</t>
@@ -31659,8 +31643,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E679" t="inlineStr"/>
-      <c r="F679" t="inlineStr"/>
       <c r="G679" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -31707,8 +31689,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E680" t="inlineStr"/>
-      <c r="F680" t="inlineStr"/>
       <c r="G680" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -31755,8 +31735,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E681" t="inlineStr"/>
-      <c r="F681" t="inlineStr"/>
       <c r="G681" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -31803,8 +31781,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E682" t="inlineStr"/>
-      <c r="F682" t="inlineStr"/>
       <c r="G682" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -31851,8 +31827,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E683" t="inlineStr"/>
-      <c r="F683" t="inlineStr"/>
       <c r="G683" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -31899,8 +31873,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E684" t="inlineStr"/>
-      <c r="F684" t="inlineStr"/>
       <c r="G684" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -31947,8 +31919,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E685" t="inlineStr"/>
-      <c r="F685" t="inlineStr"/>
       <c r="G685" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -31995,8 +31965,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E686" t="inlineStr"/>
-      <c r="F686" t="inlineStr"/>
       <c r="G686" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -32043,8 +32011,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E687" t="inlineStr"/>
-      <c r="F687" t="inlineStr"/>
       <c r="G687" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -32091,8 +32057,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E688" t="inlineStr"/>
-      <c r="F688" t="inlineStr"/>
       <c r="G688" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -32139,8 +32103,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E689" t="inlineStr"/>
-      <c r="F689" t="inlineStr"/>
       <c r="G689" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -32187,8 +32149,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E690" t="inlineStr"/>
-      <c r="F690" t="inlineStr"/>
       <c r="G690" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -32235,8 +32195,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E691" t="inlineStr"/>
-      <c r="F691" t="inlineStr"/>
       <c r="G691" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -32283,8 +32241,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E692" t="inlineStr"/>
-      <c r="F692" t="inlineStr"/>
       <c r="G692" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -32331,8 +32287,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E693" t="inlineStr"/>
-      <c r="F693" t="inlineStr"/>
       <c r="G693" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -32379,8 +32333,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E694" t="inlineStr"/>
-      <c r="F694" t="inlineStr"/>
       <c r="G694" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -32427,8 +32379,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E695" t="inlineStr"/>
-      <c r="F695" t="inlineStr"/>
       <c r="G695" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -32475,8 +32425,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E696" t="inlineStr"/>
-      <c r="F696" t="inlineStr"/>
       <c r="G696" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -32523,8 +32471,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E697" t="inlineStr"/>
-      <c r="F697" t="inlineStr"/>
       <c r="G697" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -32571,8 +32517,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E698" t="inlineStr"/>
-      <c r="F698" t="inlineStr"/>
       <c r="G698" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -32619,8 +32563,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E699" t="inlineStr"/>
-      <c r="F699" t="inlineStr"/>
       <c r="G699" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -32667,8 +32609,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E700" t="inlineStr"/>
-      <c r="F700" t="inlineStr"/>
       <c r="G700" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -32715,8 +32655,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E701" t="inlineStr"/>
-      <c r="F701" t="inlineStr"/>
       <c r="G701" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -32763,8 +32701,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E702" t="inlineStr"/>
-      <c r="F702" t="inlineStr"/>
       <c r="G702" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -32811,8 +32747,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E703" t="inlineStr"/>
-      <c r="F703" t="inlineStr"/>
       <c r="G703" t="inlineStr">
         <is>
           <t>4-3</t>
@@ -32859,8 +32793,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E704" t="inlineStr"/>
-      <c r="F704" t="inlineStr"/>
       <c r="G704" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -32881,6 +32813,2118 @@
         <v>0</v>
       </c>
       <c r="L704" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>FC Utrecht vs Go Ahead Eagles</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>FC Utrecht</t>
+        </is>
+      </c>
+      <c r="D705" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E705" t="inlineStr"/>
+      <c r="F705" t="inlineStr"/>
+      <c r="G705" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H705" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I705" t="n">
+        <v>0</v>
+      </c>
+      <c r="J705" t="n">
+        <v>0</v>
+      </c>
+      <c r="K705" t="n">
+        <v>0</v>
+      </c>
+      <c r="L705" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Al Ettifaq vs Al Faisaly</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Al Ettifaq</t>
+        </is>
+      </c>
+      <c r="D706" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E706" t="inlineStr"/>
+      <c r="F706" t="inlineStr"/>
+      <c r="G706" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H706" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I706" t="n">
+        <v>0</v>
+      </c>
+      <c r="J706" t="n">
+        <v>0</v>
+      </c>
+      <c r="K706" t="n">
+        <v>0</v>
+      </c>
+      <c r="L706" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>AEK Athens vs LASK Linz</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>AEK Athens</t>
+        </is>
+      </c>
+      <c r="D707" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E707" t="inlineStr"/>
+      <c r="F707" t="inlineStr"/>
+      <c r="G707" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H707" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I707" t="n">
+        <v>0</v>
+      </c>
+      <c r="J707" t="n">
+        <v>0</v>
+      </c>
+      <c r="K707" t="n">
+        <v>0</v>
+      </c>
+      <c r="L707" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Club Brugge vs Aston Villa</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Aston Villa</t>
+        </is>
+      </c>
+      <c r="D708" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E708" t="inlineStr"/>
+      <c r="F708" t="inlineStr"/>
+      <c r="G708" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H708" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I708" t="n">
+        <v>0</v>
+      </c>
+      <c r="J708" t="n">
+        <v>0</v>
+      </c>
+      <c r="K708" t="n">
+        <v>0</v>
+      </c>
+      <c r="L708" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>NEC Nijmegen vs Excelsior</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>NEC Nijmegen</t>
+        </is>
+      </c>
+      <c r="D709" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E709" t="inlineStr"/>
+      <c r="F709" t="inlineStr"/>
+      <c r="G709" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H709" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I709" t="n">
+        <v>0</v>
+      </c>
+      <c r="J709" t="n">
+        <v>0</v>
+      </c>
+      <c r="K709" t="n">
+        <v>0</v>
+      </c>
+      <c r="L709" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Doncaster Rovers vs Huddersfield Town</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Huddersfield Town</t>
+        </is>
+      </c>
+      <c r="D710" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E710" t="inlineStr"/>
+      <c r="F710" t="inlineStr"/>
+      <c r="G710" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H710" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I710" t="n">
+        <v>0</v>
+      </c>
+      <c r="J710" t="n">
+        <v>0</v>
+      </c>
+      <c r="K710" t="n">
+        <v>0</v>
+      </c>
+      <c r="L710" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Exeter City vs Tottenham Hotspur U21</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Exeter City</t>
+        </is>
+      </c>
+      <c r="D711" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E711" t="inlineStr"/>
+      <c r="F711" t="inlineStr"/>
+      <c r="G711" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H711" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I711" t="n">
+        <v>0</v>
+      </c>
+      <c r="J711" t="n">
+        <v>0</v>
+      </c>
+      <c r="K711" t="n">
+        <v>0</v>
+      </c>
+      <c r="L711" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Al Ittihad vs Al Fayha</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Al Ittihad</t>
+        </is>
+      </c>
+      <c r="D712" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E712" t="inlineStr"/>
+      <c r="F712" t="inlineStr"/>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H712" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I712" t="n">
+        <v>0</v>
+      </c>
+      <c r="J712" t="n">
+        <v>0</v>
+      </c>
+      <c r="K712" t="n">
+        <v>0</v>
+      </c>
+      <c r="L712" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Al Qadsiah vs Al Ahli</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Al Qadsiah</t>
+        </is>
+      </c>
+      <c r="D713" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E713" t="inlineStr"/>
+      <c r="F713" t="inlineStr"/>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H713" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I713" t="n">
+        <v>0</v>
+      </c>
+      <c r="J713" t="n">
+        <v>0</v>
+      </c>
+      <c r="K713" t="n">
+        <v>0</v>
+      </c>
+      <c r="L713" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Blackburn Rovers vs Sheffield United</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Sheffield United</t>
+        </is>
+      </c>
+      <c r="D714" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E714" t="inlineStr"/>
+      <c r="F714" t="inlineStr"/>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H714" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I714" t="n">
+        <v>0</v>
+      </c>
+      <c r="J714" t="n">
+        <v>0</v>
+      </c>
+      <c r="K714" t="n">
+        <v>0</v>
+      </c>
+      <c r="L714" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Cardiff City vs Stoke City</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>Cardiff City</t>
+        </is>
+      </c>
+      <c r="D715" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E715" t="inlineStr"/>
+      <c r="F715" t="inlineStr"/>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H715" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I715" t="n">
+        <v>0</v>
+      </c>
+      <c r="J715" t="n">
+        <v>0</v>
+      </c>
+      <c r="K715" t="n">
+        <v>0</v>
+      </c>
+      <c r="L715" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Southampton vs Swansea City</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Southampton</t>
+        </is>
+      </c>
+      <c r="D716" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E716" t="inlineStr"/>
+      <c r="F716" t="inlineStr"/>
+      <c r="G716" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I716" t="n">
+        <v>0</v>
+      </c>
+      <c r="J716" t="n">
+        <v>0</v>
+      </c>
+      <c r="K716" t="n">
+        <v>0</v>
+      </c>
+      <c r="L716" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Watford vs Preston North End</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="D717" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E717" t="inlineStr"/>
+      <c r="F717" t="inlineStr"/>
+      <c r="G717" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I717" t="n">
+        <v>0</v>
+      </c>
+      <c r="J717" t="n">
+        <v>0</v>
+      </c>
+      <c r="K717" t="n">
+        <v>0</v>
+      </c>
+      <c r="L717" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Wrexham vs Burnley</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Wrexham</t>
+        </is>
+      </c>
+      <c r="D718" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E718" t="inlineStr"/>
+      <c r="F718" t="inlineStr"/>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H718" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I718" t="n">
+        <v>0</v>
+      </c>
+      <c r="J718" t="n">
+        <v>0</v>
+      </c>
+      <c r="K718" t="n">
+        <v>0</v>
+      </c>
+      <c r="L718" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>AFC Bournemouth vs Lincoln City</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>AFC Bournemouth</t>
+        </is>
+      </c>
+      <c r="D719" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E719" t="inlineStr"/>
+      <c r="F719" t="inlineStr"/>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H719" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I719" t="n">
+        <v>0</v>
+      </c>
+      <c r="J719" t="n">
+        <v>0</v>
+      </c>
+      <c r="K719" t="n">
+        <v>0</v>
+      </c>
+      <c r="L719" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Crystal Palace vs Middlesbrough</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Crystal Palace</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E720" t="inlineStr"/>
+      <c r="F720" t="inlineStr"/>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H720" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I720" t="n">
+        <v>0</v>
+      </c>
+      <c r="J720" t="n">
+        <v>0</v>
+      </c>
+      <c r="K720" t="n">
+        <v>0</v>
+      </c>
+      <c r="L720" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Leyton Orient vs Bradford City</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>Bradford City</t>
+        </is>
+      </c>
+      <c r="D721" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E721" t="inlineStr"/>
+      <c r="F721" t="inlineStr"/>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H721" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I721" t="n">
+        <v>0</v>
+      </c>
+      <c r="J721" t="n">
+        <v>0</v>
+      </c>
+      <c r="K721" t="n">
+        <v>0</v>
+      </c>
+      <c r="L721" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Sunderland vs Hull City</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Sunderland</t>
+        </is>
+      </c>
+      <c r="D722" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E722" t="inlineStr"/>
+      <c r="F722" t="inlineStr"/>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H722" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I722" t="n">
+        <v>0</v>
+      </c>
+      <c r="J722" t="n">
+        <v>0</v>
+      </c>
+      <c r="K722" t="n">
+        <v>0</v>
+      </c>
+      <c r="L722" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Hitchin Town vs Biggleswade Town</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Hitchin Town</t>
+        </is>
+      </c>
+      <c r="D723" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E723" t="inlineStr"/>
+      <c r="F723" t="inlineStr"/>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H723" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I723" t="n">
+        <v>0</v>
+      </c>
+      <c r="J723" t="n">
+        <v>0</v>
+      </c>
+      <c r="K723" t="n">
+        <v>0</v>
+      </c>
+      <c r="L723" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Needham Market vs Stanway Rovers FC</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Needham Market</t>
+        </is>
+      </c>
+      <c r="D724" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E724" t="inlineStr"/>
+      <c r="F724" t="inlineStr"/>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H724" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I724" t="n">
+        <v>0</v>
+      </c>
+      <c r="J724" t="n">
+        <v>0</v>
+      </c>
+      <c r="K724" t="n">
+        <v>0</v>
+      </c>
+      <c r="L724" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Worcester City vs Knowle</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Worcester City</t>
+        </is>
+      </c>
+      <c r="D725" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E725" t="inlineStr"/>
+      <c r="F725" t="inlineStr"/>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H725" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I725" t="n">
+        <v>0</v>
+      </c>
+      <c r="J725" t="n">
+        <v>0</v>
+      </c>
+      <c r="K725" t="n">
+        <v>0</v>
+      </c>
+      <c r="L725" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Annan Athletic vs Motherwell B</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Annan Athletic</t>
+        </is>
+      </c>
+      <c r="D726" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E726" t="inlineStr"/>
+      <c r="F726" t="inlineStr"/>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H726" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I726" t="n">
+        <v>0</v>
+      </c>
+      <c r="J726" t="n">
+        <v>0</v>
+      </c>
+      <c r="K726" t="n">
+        <v>0</v>
+      </c>
+      <c r="L726" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Banks O'Dee vs Forfar Athletic</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Forfar Athletic</t>
+        </is>
+      </c>
+      <c r="D727" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E727" t="inlineStr"/>
+      <c r="F727" t="inlineStr"/>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H727" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I727" t="n">
+        <v>0</v>
+      </c>
+      <c r="J727" t="n">
+        <v>0</v>
+      </c>
+      <c r="K727" t="n">
+        <v>0</v>
+      </c>
+      <c r="L727" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Berwick Rangers vs Hibernian B</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>Berwick Rangers</t>
+        </is>
+      </c>
+      <c r="D728" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E728" t="inlineStr"/>
+      <c r="F728" t="inlineStr"/>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H728" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I728" t="n">
+        <v>0</v>
+      </c>
+      <c r="J728" t="n">
+        <v>0</v>
+      </c>
+      <c r="K728" t="n">
+        <v>0</v>
+      </c>
+      <c r="L728" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Clyde vs East Fife</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>East Fife</t>
+        </is>
+      </c>
+      <c r="D729" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E729" t="inlineStr"/>
+      <c r="F729" t="inlineStr"/>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H729" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I729" t="n">
+        <v>0</v>
+      </c>
+      <c r="J729" t="n">
+        <v>0</v>
+      </c>
+      <c r="K729" t="n">
+        <v>0</v>
+      </c>
+      <c r="L729" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Clydebank vs Alloa Athletic</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Alloa Athletic</t>
+        </is>
+      </c>
+      <c r="D730" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E730" t="inlineStr"/>
+      <c r="F730" t="inlineStr"/>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H730" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I730" t="n">
+        <v>0</v>
+      </c>
+      <c r="J730" t="n">
+        <v>0</v>
+      </c>
+      <c r="K730" t="n">
+        <v>0</v>
+      </c>
+      <c r="L730" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Cove Rangers vs Dumbarton</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Cove Rangers</t>
+        </is>
+      </c>
+      <c r="D731" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E731" t="inlineStr"/>
+      <c r="F731" t="inlineStr"/>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>6-1</t>
+        </is>
+      </c>
+      <c r="H731" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I731" t="n">
+        <v>0</v>
+      </c>
+      <c r="J731" t="n">
+        <v>0</v>
+      </c>
+      <c r="K731" t="n">
+        <v>0</v>
+      </c>
+      <c r="L731" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Cowdenbeath vs Kilmarnock B</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Cowdenbeath</t>
+        </is>
+      </c>
+      <c r="D732" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E732" t="inlineStr"/>
+      <c r="F732" t="inlineStr"/>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H732" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I732" t="n">
+        <v>0</v>
+      </c>
+      <c r="J732" t="n">
+        <v>0</v>
+      </c>
+      <c r="K732" t="n">
+        <v>0</v>
+      </c>
+      <c r="L732" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Cumbernauld Colts vs Kelty Hearts</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Kelty Hearts</t>
+        </is>
+      </c>
+      <c r="D733" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E733" t="inlineStr"/>
+      <c r="F733" t="inlineStr"/>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H733" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I733" t="n">
+        <v>0</v>
+      </c>
+      <c r="J733" t="n">
+        <v>0</v>
+      </c>
+      <c r="K733" t="n">
+        <v>0</v>
+      </c>
+      <c r="L733" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>East Kilbride vs Bonnyrigg Rose</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>East Kilbride</t>
+        </is>
+      </c>
+      <c r="D734" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E734" t="inlineStr"/>
+      <c r="F734" t="inlineStr"/>
+      <c r="G734" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I734" t="n">
+        <v>0</v>
+      </c>
+      <c r="J734" t="n">
+        <v>0</v>
+      </c>
+      <c r="K734" t="n">
+        <v>0</v>
+      </c>
+      <c r="L734" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Edinburgh City vs Queen of the South</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>Queen of the South</t>
+        </is>
+      </c>
+      <c r="D735" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E735" t="inlineStr"/>
+      <c r="F735" t="inlineStr"/>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H735" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I735" t="n">
+        <v>0</v>
+      </c>
+      <c r="J735" t="n">
+        <v>0</v>
+      </c>
+      <c r="K735" t="n">
+        <v>0</v>
+      </c>
+      <c r="L735" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund vs Villarreal</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Borussia Dortmund</t>
+        </is>
+      </c>
+      <c r="D736" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E736" t="inlineStr"/>
+      <c r="F736" t="inlineStr"/>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H736" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I736" t="n">
+        <v>0</v>
+      </c>
+      <c r="J736" t="n">
+        <v>0</v>
+      </c>
+      <c r="K736" t="n">
+        <v>0</v>
+      </c>
+      <c r="L736" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>FC Porto vs Manchester City</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Manchester City</t>
+        </is>
+      </c>
+      <c r="D737" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E737" t="inlineStr"/>
+      <c r="F737" t="inlineStr"/>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H737" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I737" t="n">
+        <v>0</v>
+      </c>
+      <c r="J737" t="n">
+        <v>0</v>
+      </c>
+      <c r="K737" t="n">
+        <v>0</v>
+      </c>
+      <c r="L737" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Lille vs Real Betis</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="D738" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E738" t="inlineStr"/>
+      <c r="F738" t="inlineStr"/>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H738" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I738" t="n">
+        <v>0</v>
+      </c>
+      <c r="J738" t="n">
+        <v>0</v>
+      </c>
+      <c r="K738" t="n">
+        <v>0</v>
+      </c>
+      <c r="L738" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Real Madrid vs Internazionale</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>Real Madrid</t>
+        </is>
+      </c>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr"/>
+      <c r="F739" t="inlineStr"/>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I739" t="n">
+        <v>0</v>
+      </c>
+      <c r="J739" t="n">
+        <v>0</v>
+      </c>
+      <c r="K739" t="n">
+        <v>0</v>
+      </c>
+      <c r="L739" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Bolton Wanderers vs West Ham United</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>West Ham United</t>
+        </is>
+      </c>
+      <c r="D740" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E740" t="inlineStr"/>
+      <c r="F740" t="inlineStr"/>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H740" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I740" t="n">
+        <v>0</v>
+      </c>
+      <c r="J740" t="n">
+        <v>0</v>
+      </c>
+      <c r="K740" t="n">
+        <v>0</v>
+      </c>
+      <c r="L740" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Millwall vs Newcastle United</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Newcastle United</t>
+        </is>
+      </c>
+      <c r="D741" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E741" t="inlineStr"/>
+      <c r="F741" t="inlineStr"/>
+      <c r="G741" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I741" t="n">
+        <v>0</v>
+      </c>
+      <c r="J741" t="n">
+        <v>0</v>
+      </c>
+      <c r="K741" t="n">
+        <v>0</v>
+      </c>
+      <c r="L741" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Independiente Santa Fe vs Vasco da Gama</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Independiente Santa Fe</t>
+        </is>
+      </c>
+      <c r="D742" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E742" t="inlineStr"/>
+      <c r="F742" t="inlineStr"/>
+      <c r="G742" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I742" t="n">
+        <v>0</v>
+      </c>
+      <c r="J742" t="n">
+        <v>0</v>
+      </c>
+      <c r="K742" t="n">
+        <v>0</v>
+      </c>
+      <c r="L742" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Aurora vs Real Potosí</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Aurora</t>
+        </is>
+      </c>
+      <c r="D743" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E743" t="inlineStr"/>
+      <c r="F743" t="inlineStr"/>
+      <c r="G743" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I743" t="n">
+        <v>0</v>
+      </c>
+      <c r="J743" t="n">
+        <v>0</v>
+      </c>
+      <c r="K743" t="n">
+        <v>0</v>
+      </c>
+      <c r="L743" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Hartford Athletic vs Colorado Springs Switchbacks FC</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Hartford Athletic</t>
+        </is>
+      </c>
+      <c r="D744" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E744" t="inlineStr"/>
+      <c r="F744" t="inlineStr"/>
+      <c r="G744" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I744" t="n">
+        <v>0</v>
+      </c>
+      <c r="J744" t="n">
+        <v>0</v>
+      </c>
+      <c r="K744" t="n">
+        <v>0</v>
+      </c>
+      <c r="L744" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Cuiabá vs Athletic</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>Cuiabá</t>
+        </is>
+      </c>
+      <c r="D745" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E745" t="inlineStr"/>
+      <c r="F745" t="inlineStr"/>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H745" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I745" t="n">
+        <v>0</v>
+      </c>
+      <c r="J745" t="n">
+        <v>0</v>
+      </c>
+      <c r="K745" t="n">
+        <v>0</v>
+      </c>
+      <c r="L745" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Criciúma vs Juventude</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Criciúma</t>
+        </is>
+      </c>
+      <c r="D746" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E746" t="inlineStr"/>
+      <c r="F746" t="inlineStr"/>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H746" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I746" t="n">
+        <v>0</v>
+      </c>
+      <c r="J746" t="n">
+        <v>0</v>
+      </c>
+      <c r="K746" t="n">
+        <v>0</v>
+      </c>
+      <c r="L746" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Boca Juniors vs São Paulo</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Boca Juniors</t>
+        </is>
+      </c>
+      <c r="D747" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E747" t="inlineStr"/>
+      <c r="F747" t="inlineStr"/>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H747" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I747" t="n">
+        <v>1</v>
+      </c>
+      <c r="J747" t="n">
+        <v>0</v>
+      </c>
+      <c r="K747" t="n">
+        <v>0</v>
+      </c>
+      <c r="L747" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Oriente Petrolero vs Guabirá</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Oriente Petrolero</t>
+        </is>
+      </c>
+      <c r="D748" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E748" t="inlineStr"/>
+      <c r="F748" t="inlineStr"/>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H748" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I748" t="n">
+        <v>0</v>
+      </c>
+      <c r="J748" t="n">
+        <v>0</v>
+      </c>
+      <c r="K748" t="n">
+        <v>0</v>
+      </c>
+      <c r="L748" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -32897,7 +34941,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33097,6 +35141,25 @@
       </c>
       <c r="E11" t="n">
         <v>34</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>44</v>
+      </c>
+      <c r="C12" t="n">
+        <v>39</v>
+      </c>
+      <c r="D12" t="n">
+        <v>88.59999999999999</v>
+      </c>
+      <c r="E12" t="n">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -33110,7 +35173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33140,6 +35203,27 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-10
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L748"/>
+  <dimension ref="A1:L797"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -32839,8 +32839,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E705" t="inlineStr"/>
-      <c r="F705" t="inlineStr"/>
       <c r="G705" t="inlineStr">
         <is>
           <t>3-3</t>
@@ -32887,8 +32885,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E706" t="inlineStr"/>
-      <c r="F706" t="inlineStr"/>
       <c r="G706" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -32935,8 +32931,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E707" t="inlineStr"/>
-      <c r="F707" t="inlineStr"/>
       <c r="G707" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -32983,8 +32977,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E708" t="inlineStr"/>
-      <c r="F708" t="inlineStr"/>
       <c r="G708" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -33031,8 +33023,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E709" t="inlineStr"/>
-      <c r="F709" t="inlineStr"/>
       <c r="G709" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -33079,8 +33069,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E710" t="inlineStr"/>
-      <c r="F710" t="inlineStr"/>
       <c r="G710" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -33127,8 +33115,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E711" t="inlineStr"/>
-      <c r="F711" t="inlineStr"/>
       <c r="G711" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -33175,8 +33161,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E712" t="inlineStr"/>
-      <c r="F712" t="inlineStr"/>
       <c r="G712" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -33223,8 +33207,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E713" t="inlineStr"/>
-      <c r="F713" t="inlineStr"/>
       <c r="G713" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -33271,8 +33253,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E714" t="inlineStr"/>
-      <c r="F714" t="inlineStr"/>
       <c r="G714" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -33319,8 +33299,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E715" t="inlineStr"/>
-      <c r="F715" t="inlineStr"/>
       <c r="G715" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -33367,8 +33345,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E716" t="inlineStr"/>
-      <c r="F716" t="inlineStr"/>
       <c r="G716" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -33415,8 +33391,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E717" t="inlineStr"/>
-      <c r="F717" t="inlineStr"/>
       <c r="G717" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -33463,8 +33437,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E718" t="inlineStr"/>
-      <c r="F718" t="inlineStr"/>
       <c r="G718" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -33511,8 +33483,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E719" t="inlineStr"/>
-      <c r="F719" t="inlineStr"/>
       <c r="G719" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -33559,8 +33529,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E720" t="inlineStr"/>
-      <c r="F720" t="inlineStr"/>
       <c r="G720" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -33607,8 +33575,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E721" t="inlineStr"/>
-      <c r="F721" t="inlineStr"/>
       <c r="G721" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -33655,8 +33621,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E722" t="inlineStr"/>
-      <c r="F722" t="inlineStr"/>
       <c r="G722" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -33703,8 +33667,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E723" t="inlineStr"/>
-      <c r="F723" t="inlineStr"/>
       <c r="G723" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -33751,8 +33713,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E724" t="inlineStr"/>
-      <c r="F724" t="inlineStr"/>
       <c r="G724" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -33799,8 +33759,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E725" t="inlineStr"/>
-      <c r="F725" t="inlineStr"/>
       <c r="G725" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -33847,8 +33805,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E726" t="inlineStr"/>
-      <c r="F726" t="inlineStr"/>
       <c r="G726" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -33895,8 +33851,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E727" t="inlineStr"/>
-      <c r="F727" t="inlineStr"/>
       <c r="G727" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -33943,8 +33897,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E728" t="inlineStr"/>
-      <c r="F728" t="inlineStr"/>
       <c r="G728" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -33991,8 +33943,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E729" t="inlineStr"/>
-      <c r="F729" t="inlineStr"/>
       <c r="G729" t="inlineStr">
         <is>
           <t>1-4</t>
@@ -34039,8 +33989,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E730" t="inlineStr"/>
-      <c r="F730" t="inlineStr"/>
       <c r="G730" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -34087,8 +34035,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E731" t="inlineStr"/>
-      <c r="F731" t="inlineStr"/>
       <c r="G731" t="inlineStr">
         <is>
           <t>6-1</t>
@@ -34135,8 +34081,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E732" t="inlineStr"/>
-      <c r="F732" t="inlineStr"/>
       <c r="G732" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -34183,8 +34127,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E733" t="inlineStr"/>
-      <c r="F733" t="inlineStr"/>
       <c r="G733" t="inlineStr">
         <is>
           <t>0-3</t>
@@ -34231,8 +34173,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E734" t="inlineStr"/>
-      <c r="F734" t="inlineStr"/>
       <c r="G734" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -34279,8 +34219,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E735" t="inlineStr"/>
-      <c r="F735" t="inlineStr"/>
       <c r="G735" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -34327,8 +34265,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E736" t="inlineStr"/>
-      <c r="F736" t="inlineStr"/>
       <c r="G736" t="inlineStr">
         <is>
           <t>3-2</t>
@@ -34375,8 +34311,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E737" t="inlineStr"/>
-      <c r="F737" t="inlineStr"/>
       <c r="G737" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -34423,8 +34357,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E738" t="inlineStr"/>
-      <c r="F738" t="inlineStr"/>
       <c r="G738" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -34471,8 +34403,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E739" t="inlineStr"/>
-      <c r="F739" t="inlineStr"/>
       <c r="G739" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -34519,8 +34449,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E740" t="inlineStr"/>
-      <c r="F740" t="inlineStr"/>
       <c r="G740" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -34567,8 +34495,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E741" t="inlineStr"/>
-      <c r="F741" t="inlineStr"/>
       <c r="G741" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -34615,8 +34541,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E742" t="inlineStr"/>
-      <c r="F742" t="inlineStr"/>
       <c r="G742" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -34663,8 +34587,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E743" t="inlineStr"/>
-      <c r="F743" t="inlineStr"/>
       <c r="G743" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -34711,8 +34633,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E744" t="inlineStr"/>
-      <c r="F744" t="inlineStr"/>
       <c r="G744" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -34759,8 +34679,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E745" t="inlineStr"/>
-      <c r="F745" t="inlineStr"/>
       <c r="G745" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -34807,8 +34725,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E746" t="inlineStr"/>
-      <c r="F746" t="inlineStr"/>
       <c r="G746" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -34855,8 +34771,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E747" t="inlineStr"/>
-      <c r="F747" t="inlineStr"/>
       <c r="G747" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -34903,8 +34817,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E748" t="inlineStr"/>
-      <c r="F748" t="inlineStr"/>
       <c r="G748" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -34925,6 +34837,2358 @@
         <v>0</v>
       </c>
       <c r="L748" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Al Kholood vs Al Shabab</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>Al Shabab</t>
+        </is>
+      </c>
+      <c r="D749" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E749" t="inlineStr"/>
+      <c r="F749" t="inlineStr"/>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H749" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I749" t="n">
+        <v>0</v>
+      </c>
+      <c r="J749" t="n">
+        <v>0</v>
+      </c>
+      <c r="K749" t="n">
+        <v>0</v>
+      </c>
+      <c r="L749" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Barcelona vs Feyenoord Rotterdam</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="D750" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E750" t="inlineStr"/>
+      <c r="F750" t="inlineStr"/>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>5-1</t>
+        </is>
+      </c>
+      <c r="H750" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I750" t="n">
+        <v>1</v>
+      </c>
+      <c r="J750" t="n">
+        <v>0</v>
+      </c>
+      <c r="K750" t="n">
+        <v>0</v>
+      </c>
+      <c r="L750" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart vs Viking FK</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>VfB Stuttgart</t>
+        </is>
+      </c>
+      <c r="D751" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E751" t="inlineStr"/>
+      <c r="F751" t="inlineStr"/>
+      <c r="G751" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H751" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I751" t="n">
+        <v>1</v>
+      </c>
+      <c r="J751" t="n">
+        <v>0</v>
+      </c>
+      <c r="K751" t="n">
+        <v>0</v>
+      </c>
+      <c r="L751" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>FC Twente vs Telstar</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>FC Twente</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr"/>
+      <c r="F752" t="inlineStr"/>
+      <c r="G752" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H752" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I752" t="n">
+        <v>1</v>
+      </c>
+      <c r="J752" t="n">
+        <v>0</v>
+      </c>
+      <c r="K752" t="n">
+        <v>0</v>
+      </c>
+      <c r="L752" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Mamelodi Sundowns vs Siwelele</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Mamelodi Sundowns</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr"/>
+      <c r="F753" t="inlineStr"/>
+      <c r="G753" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H753" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I753" t="n">
+        <v>0</v>
+      </c>
+      <c r="J753" t="n">
+        <v>0</v>
+      </c>
+      <c r="K753" t="n">
+        <v>0</v>
+      </c>
+      <c r="L753" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Al Fateh vs Al Diriyah</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Al Diriyah</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr"/>
+      <c r="F754" t="inlineStr"/>
+      <c r="G754" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H754" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I754" t="n">
+        <v>0</v>
+      </c>
+      <c r="J754" t="n">
+        <v>0</v>
+      </c>
+      <c r="K754" t="n">
+        <v>0</v>
+      </c>
+      <c r="L754" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Al Nassr vs Abha</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Al Nassr</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr"/>
+      <c r="F755" t="inlineStr"/>
+      <c r="G755" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H755" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I755" t="n">
+        <v>0</v>
+      </c>
+      <c r="J755" t="n">
+        <v>0</v>
+      </c>
+      <c r="K755" t="n">
+        <v>0</v>
+      </c>
+      <c r="L755" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Defensores de Belgrano vs Los Andes</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Defensores de Belgrano</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr"/>
+      <c r="F756" t="inlineStr"/>
+      <c r="G756" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H756" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I756" t="n">
+        <v>0</v>
+      </c>
+      <c r="J756" t="n">
+        <v>0</v>
+      </c>
+      <c r="K756" t="n">
+        <v>0</v>
+      </c>
+      <c r="L756" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Derby County vs West Bromwich Albion</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>West Bromwich Albion</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr"/>
+      <c r="F757" t="inlineStr"/>
+      <c r="G757" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H757" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I757" t="n">
+        <v>0</v>
+      </c>
+      <c r="J757" t="n">
+        <v>0</v>
+      </c>
+      <c r="K757" t="n">
+        <v>0</v>
+      </c>
+      <c r="L757" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Norwich City vs Birmingham City</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr"/>
+      <c r="F758" t="inlineStr"/>
+      <c r="G758" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H758" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I758" t="n">
+        <v>0</v>
+      </c>
+      <c r="J758" t="n">
+        <v>0</v>
+      </c>
+      <c r="K758" t="n">
+        <v>0</v>
+      </c>
+      <c r="L758" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Rangers vs St Mirren</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Rangers</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr"/>
+      <c r="F759" t="inlineStr"/>
+      <c r="G759" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H759" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I759" t="n">
+        <v>0</v>
+      </c>
+      <c r="J759" t="n">
+        <v>0</v>
+      </c>
+      <c r="K759" t="n">
+        <v>0</v>
+      </c>
+      <c r="L759" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Exmouth Town vs Banbury United</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Banbury United</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr"/>
+      <c r="F760" t="inlineStr"/>
+      <c r="G760" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H760" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I760" t="n">
+        <v>0</v>
+      </c>
+      <c r="J760" t="n">
+        <v>0</v>
+      </c>
+      <c r="K760" t="n">
+        <v>0</v>
+      </c>
+      <c r="L760" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Bishop Auckland vs Emley AFC</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Emley AFC</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr"/>
+      <c r="F761" t="inlineStr"/>
+      <c r="G761" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H761" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I761" t="n">
+        <v>0</v>
+      </c>
+      <c r="J761" t="n">
+        <v>0</v>
+      </c>
+      <c r="K761" t="n">
+        <v>0</v>
+      </c>
+      <c r="L761" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Liverpool vs Atlético Madrid</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Liverpool</t>
+        </is>
+      </c>
+      <c r="D762" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E762" t="inlineStr"/>
+      <c r="F762" t="inlineStr"/>
+      <c r="G762" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H762" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I762" t="n">
+        <v>0</v>
+      </c>
+      <c r="J762" t="n">
+        <v>0</v>
+      </c>
+      <c r="K762" t="n">
+        <v>0</v>
+      </c>
+      <c r="L762" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Napoli vs Arsenal</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Arsenal</t>
+        </is>
+      </c>
+      <c r="D763" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E763" t="inlineStr"/>
+      <c r="F763" t="inlineStr"/>
+      <c r="G763" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H763" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I763" t="n">
+        <v>0</v>
+      </c>
+      <c r="J763" t="n">
+        <v>0</v>
+      </c>
+      <c r="K763" t="n">
+        <v>0</v>
+      </c>
+      <c r="L763" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain vs Slovan Bratislava</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Paris Saint-Germain</t>
+        </is>
+      </c>
+      <c r="D764" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E764" t="inlineStr"/>
+      <c r="F764" t="inlineStr"/>
+      <c r="G764" t="inlineStr">
+        <is>
+          <t>6-1</t>
+        </is>
+      </c>
+      <c r="H764" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I764" t="n">
+        <v>0</v>
+      </c>
+      <c r="J764" t="n">
+        <v>0</v>
+      </c>
+      <c r="K764" t="n">
+        <v>0</v>
+      </c>
+      <c r="L764" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Sporting CP vs Galatasaray</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Sporting CP</t>
+        </is>
+      </c>
+      <c r="D765" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E765" t="inlineStr"/>
+      <c r="F765" t="inlineStr"/>
+      <c r="G765" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H765" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I765" t="n">
+        <v>0</v>
+      </c>
+      <c r="J765" t="n">
+        <v>0</v>
+      </c>
+      <c r="K765" t="n">
+        <v>0</v>
+      </c>
+      <c r="L765" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Charlton Athletic vs Queens Park Rangers</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>Queens Park Rangers</t>
+        </is>
+      </c>
+      <c r="D766" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E766" t="inlineStr"/>
+      <c r="F766" t="inlineStr"/>
+      <c r="G766" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H766" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I766" t="n">
+        <v>0</v>
+      </c>
+      <c r="J766" t="n">
+        <v>0</v>
+      </c>
+      <c r="K766" t="n">
+        <v>0</v>
+      </c>
+      <c r="L766" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>St Johnstone vs Celtic</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Celtic</t>
+        </is>
+      </c>
+      <c r="D767" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E767" t="inlineStr"/>
+      <c r="F767" t="inlineStr"/>
+      <c r="G767" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H767" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I767" t="n">
+        <v>0</v>
+      </c>
+      <c r="J767" t="n">
+        <v>0</v>
+      </c>
+      <c r="K767" t="n">
+        <v>0</v>
+      </c>
+      <c r="L767" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Real Oruro vs Nacional Potosí</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Nacional Potosí</t>
+        </is>
+      </c>
+      <c r="D768" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E768" t="inlineStr"/>
+      <c r="F768" t="inlineStr"/>
+      <c r="G768" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H768" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I768" t="n">
+        <v>0</v>
+      </c>
+      <c r="J768" t="n">
+        <v>0</v>
+      </c>
+      <c r="K768" t="n">
+        <v>0</v>
+      </c>
+      <c r="L768" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Chelsea vs Leeds United</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Chelsea</t>
+        </is>
+      </c>
+      <c r="D769" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E769" t="inlineStr"/>
+      <c r="F769" t="inlineStr"/>
+      <c r="G769" t="inlineStr">
+        <is>
+          <t>6-3</t>
+        </is>
+      </c>
+      <c r="H769" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I769" t="n">
+        <v>0</v>
+      </c>
+      <c r="J769" t="n">
+        <v>0</v>
+      </c>
+      <c r="K769" t="n">
+        <v>0</v>
+      </c>
+      <c r="L769" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Moreirense vs Benfica</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>Benfica</t>
+        </is>
+      </c>
+      <c r="D770" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E770" t="inlineStr"/>
+      <c r="F770" t="inlineStr"/>
+      <c r="G770" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H770" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I770" t="n">
+        <v>0</v>
+      </c>
+      <c r="J770" t="n">
+        <v>0</v>
+      </c>
+      <c r="K770" t="n">
+        <v>0</v>
+      </c>
+      <c r="L770" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>C.D. Platense vs Isidro Metapán</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Isidro Metapán</t>
+        </is>
+      </c>
+      <c r="D771" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E771" t="inlineStr"/>
+      <c r="F771" t="inlineStr"/>
+      <c r="G771" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H771" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I771" t="n">
+        <v>0</v>
+      </c>
+      <c r="J771" t="n">
+        <v>0</v>
+      </c>
+      <c r="K771" t="n">
+        <v>0</v>
+      </c>
+      <c r="L771" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Deportivo San Pedro vs Deportivo Mixco</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Deportivo San Pedro</t>
+        </is>
+      </c>
+      <c r="D772" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E772" t="inlineStr"/>
+      <c r="F772" t="inlineStr"/>
+      <c r="G772" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H772" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I772" t="n">
+        <v>0</v>
+      </c>
+      <c r="J772" t="n">
+        <v>0</v>
+      </c>
+      <c r="K772" t="n">
+        <v>0</v>
+      </c>
+      <c r="L772" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Santos vs Atlético-MG</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Santos</t>
+        </is>
+      </c>
+      <c r="D773" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E773" t="inlineStr"/>
+      <c r="F773" t="inlineStr"/>
+      <c r="G773" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H773" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I773" t="n">
+        <v>0</v>
+      </c>
+      <c r="J773" t="n">
+        <v>0</v>
+      </c>
+      <c r="K773" t="n">
+        <v>0</v>
+      </c>
+      <c r="L773" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Fortaleza vs Avaí</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="D774" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E774" t="inlineStr"/>
+      <c r="F774" t="inlineStr"/>
+      <c r="G774" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H774" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I774" t="n">
+        <v>0</v>
+      </c>
+      <c r="J774" t="n">
+        <v>0</v>
+      </c>
+      <c r="K774" t="n">
+        <v>0</v>
+      </c>
+      <c r="L774" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Universitario de Vinto vs The Strongest</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>The Strongest</t>
+        </is>
+      </c>
+      <c r="D775" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E775" t="inlineStr"/>
+      <c r="F775" t="inlineStr"/>
+      <c r="G775" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H775" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I775" t="n">
+        <v>0</v>
+      </c>
+      <c r="J775" t="n">
+        <v>0</v>
+      </c>
+      <c r="K775" t="n">
+        <v>0</v>
+      </c>
+      <c r="L775" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Botafogo-SP vs Novorizontino</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Novorizontino</t>
+        </is>
+      </c>
+      <c r="D776" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E776" t="inlineStr"/>
+      <c r="F776" t="inlineStr"/>
+      <c r="G776" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H776" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I776" t="n">
+        <v>0</v>
+      </c>
+      <c r="J776" t="n">
+        <v>0</v>
+      </c>
+      <c r="K776" t="n">
+        <v>0</v>
+      </c>
+      <c r="L776" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>América de Cali vs Deportivo Pereira</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>América de Cali</t>
+        </is>
+      </c>
+      <c r="D777" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E777" t="inlineStr"/>
+      <c r="F777" t="inlineStr"/>
+      <c r="G777" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H777" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I777" t="n">
+        <v>0</v>
+      </c>
+      <c r="J777" t="n">
+        <v>0</v>
+      </c>
+      <c r="K777" t="n">
+        <v>0</v>
+      </c>
+      <c r="L777" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Atlanta United FC vs Orlando City SC</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Atlanta United FC</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr"/>
+      <c r="F778" t="inlineStr"/>
+      <c r="G778" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H778" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I778" t="n">
+        <v>0</v>
+      </c>
+      <c r="J778" t="n">
+        <v>0</v>
+      </c>
+      <c r="K778" t="n">
+        <v>0</v>
+      </c>
+      <c r="L778" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Toronto FC vs Nashville SC</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Nashville SC</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr"/>
+      <c r="F779" t="inlineStr"/>
+      <c r="G779" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H779" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I779" t="n">
+        <v>2</v>
+      </c>
+      <c r="J779" t="n">
+        <v>0</v>
+      </c>
+      <c r="K779" t="n">
+        <v>0</v>
+      </c>
+      <c r="L779" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>CF Montréal vs Charlotte FC</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>CF Montréal</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr"/>
+      <c r="F780" t="inlineStr"/>
+      <c r="G780" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H780" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I780" t="n">
+        <v>4</v>
+      </c>
+      <c r="J780" t="n">
+        <v>0</v>
+      </c>
+      <c r="K780" t="n">
+        <v>0</v>
+      </c>
+      <c r="L780" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Operário PR vs CRB</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>Operário PR</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr"/>
+      <c r="F781" t="inlineStr"/>
+      <c r="G781" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H781" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I781" t="n">
+        <v>2</v>
+      </c>
+      <c r="J781" t="n">
+        <v>0</v>
+      </c>
+      <c r="K781" t="n">
+        <v>0</v>
+      </c>
+      <c r="L781" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Philadelphia Union vs FC Cincinnati</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Philadelphia Union</t>
+        </is>
+      </c>
+      <c r="D782" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E782" t="inlineStr"/>
+      <c r="F782" t="inlineStr"/>
+      <c r="G782" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H782" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I782" t="n">
+        <v>4</v>
+      </c>
+      <c r="J782" t="n">
+        <v>0</v>
+      </c>
+      <c r="K782" t="n">
+        <v>0</v>
+      </c>
+      <c r="L782" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>New York City FC vs New England Revolution</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>New York City FC</t>
+        </is>
+      </c>
+      <c r="D783" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E783" t="inlineStr"/>
+      <c r="F783" t="inlineStr"/>
+      <c r="G783" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H783" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I783" t="n">
+        <v>0</v>
+      </c>
+      <c r="J783" t="n">
+        <v>0</v>
+      </c>
+      <c r="K783" t="n">
+        <v>0</v>
+      </c>
+      <c r="L783" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Once Caldas vs Alianza FC</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Once Caldas</t>
+        </is>
+      </c>
+      <c r="D784" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E784" t="inlineStr"/>
+      <c r="F784" t="inlineStr"/>
+      <c r="G784" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H784" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I784" t="n">
+        <v>0</v>
+      </c>
+      <c r="J784" t="n">
+        <v>0</v>
+      </c>
+      <c r="K784" t="n">
+        <v>0</v>
+      </c>
+      <c r="L784" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Comunicaciones vs Marquense</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="D785" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E785" t="inlineStr"/>
+      <c r="F785" t="inlineStr"/>
+      <c r="G785" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H785" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I785" t="n">
+        <v>0</v>
+      </c>
+      <c r="J785" t="n">
+        <v>0</v>
+      </c>
+      <c r="K785" t="n">
+        <v>0</v>
+      </c>
+      <c r="L785" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Chicago Fire FC vs Inter Miami CF</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Chicago Fire FC</t>
+        </is>
+      </c>
+      <c r="D786" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E786" t="inlineStr"/>
+      <c r="F786" t="inlineStr"/>
+      <c r="G786" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H786" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I786" t="n">
+        <v>6</v>
+      </c>
+      <c r="J786" t="n">
+        <v>0</v>
+      </c>
+      <c r="K786" t="n">
+        <v>0</v>
+      </c>
+      <c r="L786" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Minnesota United FC vs FC Dallas</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Minnesota United FC</t>
+        </is>
+      </c>
+      <c r="D787" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E787" t="inlineStr"/>
+      <c r="F787" t="inlineStr"/>
+      <c r="G787" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H787" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I787" t="n">
+        <v>4</v>
+      </c>
+      <c r="J787" t="n">
+        <v>0</v>
+      </c>
+      <c r="K787" t="n">
+        <v>0</v>
+      </c>
+      <c r="L787" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Houston Dynamo FC vs Real Salt Lake</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Houston Dynamo FC</t>
+        </is>
+      </c>
+      <c r="D788" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E788" t="inlineStr"/>
+      <c r="F788" t="inlineStr"/>
+      <c r="G788" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H788" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I788" t="n">
+        <v>3</v>
+      </c>
+      <c r="J788" t="n">
+        <v>0</v>
+      </c>
+      <c r="K788" t="n">
+        <v>0</v>
+      </c>
+      <c r="L788" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Corinthians</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="D789" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E789" t="inlineStr"/>
+      <c r="F789" t="inlineStr"/>
+      <c r="G789" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H789" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I789" t="n">
+        <v>1</v>
+      </c>
+      <c r="J789" t="n">
+        <v>0</v>
+      </c>
+      <c r="K789" t="n">
+        <v>0</v>
+      </c>
+      <c r="L789" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Atlético Goianiense vs Ceará</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Atlético Goianiense</t>
+        </is>
+      </c>
+      <c r="D790" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E790" t="inlineStr"/>
+      <c r="F790" t="inlineStr"/>
+      <c r="G790" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H790" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I790" t="n">
+        <v>5</v>
+      </c>
+      <c r="J790" t="n">
+        <v>0</v>
+      </c>
+      <c r="K790" t="n">
+        <v>0</v>
+      </c>
+      <c r="L790" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>CD Municipal Limeño vs Águila</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>Águila</t>
+        </is>
+      </c>
+      <c r="D791" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E791" t="inlineStr"/>
+      <c r="F791" t="inlineStr"/>
+      <c r="G791" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H791" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I791" t="n">
+        <v>0</v>
+      </c>
+      <c r="J791" t="n">
+        <v>0</v>
+      </c>
+      <c r="K791" t="n">
+        <v>0</v>
+      </c>
+      <c r="L791" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Saprissa vs Cartaginés</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Saprissa</t>
+        </is>
+      </c>
+      <c r="D792" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E792" t="inlineStr"/>
+      <c r="F792" t="inlineStr"/>
+      <c r="G792" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H792" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I792" t="n">
+        <v>0</v>
+      </c>
+      <c r="J792" t="n">
+        <v>0</v>
+      </c>
+      <c r="K792" t="n">
+        <v>0</v>
+      </c>
+      <c r="L792" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Deportivo Pasto vs Independiente Medellín</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Independiente Medellín</t>
+        </is>
+      </c>
+      <c r="D793" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E793" t="inlineStr"/>
+      <c r="F793" t="inlineStr"/>
+      <c r="G793" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H793" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I793" t="n">
+        <v>0</v>
+      </c>
+      <c r="J793" t="n">
+        <v>0</v>
+      </c>
+      <c r="K793" t="n">
+        <v>0</v>
+      </c>
+      <c r="L793" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Suchitepequez vs CD Guastatoya</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Suchitepequez</t>
+        </is>
+      </c>
+      <c r="D794" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E794" t="inlineStr"/>
+      <c r="F794" t="inlineStr"/>
+      <c r="G794" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H794" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I794" t="n">
+        <v>0</v>
+      </c>
+      <c r="J794" t="n">
+        <v>0</v>
+      </c>
+      <c r="K794" t="n">
+        <v>0</v>
+      </c>
+      <c r="L794" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>San Diego FC vs San Jose Earthquakes</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>San Diego FC</t>
+        </is>
+      </c>
+      <c r="D795" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E795" t="inlineStr"/>
+      <c r="F795" t="inlineStr"/>
+      <c r="G795" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H795" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I795" t="n">
+        <v>1</v>
+      </c>
+      <c r="J795" t="n">
+        <v>0</v>
+      </c>
+      <c r="K795" t="n">
+        <v>0</v>
+      </c>
+      <c r="L795" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Portland Timbers vs St. Louis CITY SC</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Portland Timbers</t>
+        </is>
+      </c>
+      <c r="D796" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E796" t="inlineStr"/>
+      <c r="F796" t="inlineStr"/>
+      <c r="G796" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H796" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I796" t="n">
+        <v>1</v>
+      </c>
+      <c r="J796" t="n">
+        <v>0</v>
+      </c>
+      <c r="K796" t="n">
+        <v>0</v>
+      </c>
+      <c r="L796" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>FC Motagua vs Alianza FC</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>FC Motagua</t>
+        </is>
+      </c>
+      <c r="D797" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E797" t="inlineStr"/>
+      <c r="F797" t="inlineStr"/>
+      <c r="G797" t="inlineStr">
+        <is>
+          <t>3-0</t>
+        </is>
+      </c>
+      <c r="H797" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I797" t="n">
+        <v>0</v>
+      </c>
+      <c r="J797" t="n">
+        <v>0</v>
+      </c>
+      <c r="K797" t="n">
+        <v>0</v>
+      </c>
+      <c r="L797" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -34941,7 +37205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35160,6 +37424,25 @@
       </c>
       <c r="E12" t="n">
         <v>44</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>49</v>
+      </c>
+      <c r="C13" t="n">
+        <v>40</v>
+      </c>
+      <c r="D13" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="E13" t="n">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -35173,7 +37456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35224,6 +37507,195 @@
         <v>0</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>11</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>18.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>value_alert</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-11
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L797"/>
+  <dimension ref="A1:L813"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -34863,8 +34863,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E749" t="inlineStr"/>
-      <c r="F749" t="inlineStr"/>
       <c r="G749" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -34911,8 +34909,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E750" t="inlineStr"/>
-      <c r="F750" t="inlineStr"/>
       <c r="G750" t="inlineStr">
         <is>
           <t>5-1</t>
@@ -34959,8 +34955,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E751" t="inlineStr"/>
-      <c r="F751" t="inlineStr"/>
       <c r="G751" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -35007,8 +35001,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E752" t="inlineStr"/>
-      <c r="F752" t="inlineStr"/>
       <c r="G752" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -35055,8 +35047,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E753" t="inlineStr"/>
-      <c r="F753" t="inlineStr"/>
       <c r="G753" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -35103,8 +35093,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E754" t="inlineStr"/>
-      <c r="F754" t="inlineStr"/>
       <c r="G754" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -35151,8 +35139,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E755" t="inlineStr"/>
-      <c r="F755" t="inlineStr"/>
       <c r="G755" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -35199,8 +35185,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E756" t="inlineStr"/>
-      <c r="F756" t="inlineStr"/>
       <c r="G756" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -35247,8 +35231,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E757" t="inlineStr"/>
-      <c r="F757" t="inlineStr"/>
       <c r="G757" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -35295,8 +35277,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E758" t="inlineStr"/>
-      <c r="F758" t="inlineStr"/>
       <c r="G758" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -35343,8 +35323,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E759" t="inlineStr"/>
-      <c r="F759" t="inlineStr"/>
       <c r="G759" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -35391,8 +35369,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E760" t="inlineStr"/>
-      <c r="F760" t="inlineStr"/>
       <c r="G760" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -35439,8 +35415,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E761" t="inlineStr"/>
-      <c r="F761" t="inlineStr"/>
       <c r="G761" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -35487,8 +35461,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E762" t="inlineStr"/>
-      <c r="F762" t="inlineStr"/>
       <c r="G762" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -35535,8 +35507,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E763" t="inlineStr"/>
-      <c r="F763" t="inlineStr"/>
       <c r="G763" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -35583,8 +35553,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E764" t="inlineStr"/>
-      <c r="F764" t="inlineStr"/>
       <c r="G764" t="inlineStr">
         <is>
           <t>6-1</t>
@@ -35631,8 +35599,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E765" t="inlineStr"/>
-      <c r="F765" t="inlineStr"/>
       <c r="G765" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -35679,8 +35645,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E766" t="inlineStr"/>
-      <c r="F766" t="inlineStr"/>
       <c r="G766" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -35727,8 +35691,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E767" t="inlineStr"/>
-      <c r="F767" t="inlineStr"/>
       <c r="G767" t="inlineStr">
         <is>
           <t>0-1</t>
@@ -35775,8 +35737,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E768" t="inlineStr"/>
-      <c r="F768" t="inlineStr"/>
       <c r="G768" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -35823,8 +35783,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E769" t="inlineStr"/>
-      <c r="F769" t="inlineStr"/>
       <c r="G769" t="inlineStr">
         <is>
           <t>6-3</t>
@@ -35871,8 +35829,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E770" t="inlineStr"/>
-      <c r="F770" t="inlineStr"/>
       <c r="G770" t="inlineStr">
         <is>
           <t>0-4</t>
@@ -35919,8 +35875,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E771" t="inlineStr"/>
-      <c r="F771" t="inlineStr"/>
       <c r="G771" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -35967,8 +35921,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E772" t="inlineStr"/>
-      <c r="F772" t="inlineStr"/>
       <c r="G772" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -36015,8 +35967,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E773" t="inlineStr"/>
-      <c r="F773" t="inlineStr"/>
       <c r="G773" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -36063,8 +36013,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E774" t="inlineStr"/>
-      <c r="F774" t="inlineStr"/>
       <c r="G774" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -36111,8 +36059,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E775" t="inlineStr"/>
-      <c r="F775" t="inlineStr"/>
       <c r="G775" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -36159,8 +36105,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E776" t="inlineStr"/>
-      <c r="F776" t="inlineStr"/>
       <c r="G776" t="inlineStr">
         <is>
           <t>1-3</t>
@@ -36207,8 +36151,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E777" t="inlineStr"/>
-      <c r="F777" t="inlineStr"/>
       <c r="G777" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -36255,8 +36197,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E778" t="inlineStr"/>
-      <c r="F778" t="inlineStr"/>
       <c r="G778" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -36303,8 +36243,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E779" t="inlineStr"/>
-      <c r="F779" t="inlineStr"/>
       <c r="G779" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -36351,8 +36289,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E780" t="inlineStr"/>
-      <c r="F780" t="inlineStr"/>
       <c r="G780" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -36399,8 +36335,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E781" t="inlineStr"/>
-      <c r="F781" t="inlineStr"/>
       <c r="G781" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -36447,8 +36381,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E782" t="inlineStr"/>
-      <c r="F782" t="inlineStr"/>
       <c r="G782" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -36495,8 +36427,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E783" t="inlineStr"/>
-      <c r="F783" t="inlineStr"/>
       <c r="G783" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -36543,8 +36473,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E784" t="inlineStr"/>
-      <c r="F784" t="inlineStr"/>
       <c r="G784" t="inlineStr">
         <is>
           <t>1-0</t>
@@ -36591,8 +36519,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E785" t="inlineStr"/>
-      <c r="F785" t="inlineStr"/>
       <c r="G785" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -36639,8 +36565,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E786" t="inlineStr"/>
-      <c r="F786" t="inlineStr"/>
       <c r="G786" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -36687,8 +36611,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E787" t="inlineStr"/>
-      <c r="F787" t="inlineStr"/>
       <c r="G787" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -36735,8 +36657,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E788" t="inlineStr"/>
-      <c r="F788" t="inlineStr"/>
       <c r="G788" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -36783,8 +36703,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E789" t="inlineStr"/>
-      <c r="F789" t="inlineStr"/>
       <c r="G789" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -36831,8 +36749,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E790" t="inlineStr"/>
-      <c r="F790" t="inlineStr"/>
       <c r="G790" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -36879,8 +36795,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E791" t="inlineStr"/>
-      <c r="F791" t="inlineStr"/>
       <c r="G791" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -36927,8 +36841,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E792" t="inlineStr"/>
-      <c r="F792" t="inlineStr"/>
       <c r="G792" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -36975,8 +36887,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E793" t="inlineStr"/>
-      <c r="F793" t="inlineStr"/>
       <c r="G793" t="inlineStr">
         <is>
           <t>1-4</t>
@@ -37023,8 +36933,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E794" t="inlineStr"/>
-      <c r="F794" t="inlineStr"/>
       <c r="G794" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -37071,8 +36979,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E795" t="inlineStr"/>
-      <c r="F795" t="inlineStr"/>
       <c r="G795" t="inlineStr">
         <is>
           <t>2-3</t>
@@ -37119,8 +37025,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E796" t="inlineStr"/>
-      <c r="F796" t="inlineStr"/>
       <c r="G796" t="inlineStr">
         <is>
           <t>2-2</t>
@@ -37167,8 +37071,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E797" t="inlineStr"/>
-      <c r="F797" t="inlineStr"/>
       <c r="G797" t="inlineStr">
         <is>
           <t>3-0</t>
@@ -37189,6 +37091,774 @@
         <v>0</v>
       </c>
       <c r="L797" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Fenerbahce vs AS Roma</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>AS Roma</t>
+        </is>
+      </c>
+      <c r="D798" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E798" t="inlineStr"/>
+      <c r="F798" t="inlineStr"/>
+      <c r="G798" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H798" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I798" t="n">
+        <v>2</v>
+      </c>
+      <c r="J798" t="n">
+        <v>0</v>
+      </c>
+      <c r="K798" t="n">
+        <v>0</v>
+      </c>
+      <c r="L798" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven vs Shakhtar Donetsk</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>PSV Eindhoven</t>
+        </is>
+      </c>
+      <c r="D799" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E799" t="inlineStr"/>
+      <c r="F799" t="inlineStr"/>
+      <c r="G799" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H799" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I799" t="n">
+        <v>4</v>
+      </c>
+      <c r="J799" t="n">
+        <v>0</v>
+      </c>
+      <c r="K799" t="n">
+        <v>0</v>
+      </c>
+      <c r="L799" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Panathinaikos vs Kifisia</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Panathinaikos</t>
+        </is>
+      </c>
+      <c r="D800" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E800" t="inlineStr"/>
+      <c r="F800" t="inlineStr"/>
+      <c r="G800" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H800" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I800" t="n">
+        <v>1</v>
+      </c>
+      <c r="J800" t="n">
+        <v>0</v>
+      </c>
+      <c r="K800" t="n">
+        <v>0</v>
+      </c>
+      <c r="L800" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Bayern Munich vs Bodo/Glimt</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>Bayern Munich</t>
+        </is>
+      </c>
+      <c r="D801" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E801" t="inlineStr"/>
+      <c r="F801" t="inlineStr"/>
+      <c r="G801" t="inlineStr">
+        <is>
+          <t>5-0</t>
+        </is>
+      </c>
+      <c r="H801" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I801" t="n">
+        <v>7</v>
+      </c>
+      <c r="J801" t="n">
+        <v>0</v>
+      </c>
+      <c r="K801" t="n">
+        <v>0</v>
+      </c>
+      <c r="L801" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Como vs RB Leipzig</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Como</t>
+        </is>
+      </c>
+      <c r="D802" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E802" t="inlineStr"/>
+      <c r="F802" t="inlineStr"/>
+      <c r="G802" t="inlineStr">
+        <is>
+          <t>4-1</t>
+        </is>
+      </c>
+      <c r="H802" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I802" t="n">
+        <v>0</v>
+      </c>
+      <c r="J802" t="n">
+        <v>0</v>
+      </c>
+      <c r="K802" t="n">
+        <v>0</v>
+      </c>
+      <c r="L802" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Manchester United vs Sabah FK</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Manchester United</t>
+        </is>
+      </c>
+      <c r="D803" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E803" t="inlineStr"/>
+      <c r="F803" t="inlineStr"/>
+      <c r="G803" t="inlineStr">
+        <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="H803" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I803" t="n">
+        <v>3</v>
+      </c>
+      <c r="J803" t="n">
+        <v>0</v>
+      </c>
+      <c r="K803" t="n">
+        <v>0</v>
+      </c>
+      <c r="L803" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Stevenage vs Luton Town</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Luton Town</t>
+        </is>
+      </c>
+      <c r="D804" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E804" t="inlineStr"/>
+      <c r="F804" t="inlineStr"/>
+      <c r="G804" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H804" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I804" t="n">
+        <v>3</v>
+      </c>
+      <c r="J804" t="n">
+        <v>0</v>
+      </c>
+      <c r="K804" t="n">
+        <v>0</v>
+      </c>
+      <c r="L804" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Estrela vs Braga</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="D805" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E805" t="inlineStr"/>
+      <c r="F805" t="inlineStr"/>
+      <c r="G805" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H805" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I805" t="n">
+        <v>2</v>
+      </c>
+      <c r="J805" t="n">
+        <v>0</v>
+      </c>
+      <c r="K805" t="n">
+        <v>0</v>
+      </c>
+      <c r="L805" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Aurora FC vs Municipal</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Municipal</t>
+        </is>
+      </c>
+      <c r="D806" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E806" t="inlineStr"/>
+      <c r="F806" t="inlineStr"/>
+      <c r="G806" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H806" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I806" t="n">
+        <v>0</v>
+      </c>
+      <c r="J806" t="n">
+        <v>0</v>
+      </c>
+      <c r="K806" t="n">
+        <v>0</v>
+      </c>
+      <c r="L806" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Vila Nova vs Goiás</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>Vila Nova</t>
+        </is>
+      </c>
+      <c r="D807" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E807" t="inlineStr"/>
+      <c r="F807" t="inlineStr"/>
+      <c r="G807" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H807" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I807" t="n">
+        <v>5</v>
+      </c>
+      <c r="J807" t="n">
+        <v>0</v>
+      </c>
+      <c r="K807" t="n">
+        <v>0</v>
+      </c>
+      <c r="L807" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Real Tomayapo vs Always Ready</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>Always Ready</t>
+        </is>
+      </c>
+      <c r="D808" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E808" t="inlineStr"/>
+      <c r="F808" t="inlineStr"/>
+      <c r="G808" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H808" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I808" t="n">
+        <v>0</v>
+      </c>
+      <c r="J808" t="n">
+        <v>0</v>
+      </c>
+      <c r="K808" t="n">
+        <v>0</v>
+      </c>
+      <c r="L808" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>São Bernardo vs Londrina</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>São Bernardo</t>
+        </is>
+      </c>
+      <c r="D809" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E809" t="inlineStr"/>
+      <c r="F809" t="inlineStr"/>
+      <c r="G809" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H809" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I809" t="n">
+        <v>2</v>
+      </c>
+      <c r="J809" t="n">
+        <v>0</v>
+      </c>
+      <c r="K809" t="n">
+        <v>0</v>
+      </c>
+      <c r="L809" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Sport vs Ponte Preta</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="D810" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E810" t="inlineStr"/>
+      <c r="F810" t="inlineStr"/>
+      <c r="G810" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H810" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I810" t="n">
+        <v>1</v>
+      </c>
+      <c r="J810" t="n">
+        <v>0</v>
+      </c>
+      <c r="K810" t="n">
+        <v>0</v>
+      </c>
+      <c r="L810" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Millonarios vs Deportivo Cali</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Millonarios</t>
+        </is>
+      </c>
+      <c r="D811" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E811" t="inlineStr"/>
+      <c r="F811" t="inlineStr"/>
+      <c r="G811" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H811" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I811" t="n">
+        <v>3</v>
+      </c>
+      <c r="J811" t="n">
+        <v>0</v>
+      </c>
+      <c r="K811" t="n">
+        <v>0</v>
+      </c>
+      <c r="L811" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>CD Malacateco vs Antigua GFC</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>CD Malacateco</t>
+        </is>
+      </c>
+      <c r="D812" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E812" t="inlineStr"/>
+      <c r="F812" t="inlineStr"/>
+      <c r="G812" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H812" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I812" t="n">
+        <v>0</v>
+      </c>
+      <c r="J812" t="n">
+        <v>0</v>
+      </c>
+      <c r="K812" t="n">
+        <v>0</v>
+      </c>
+      <c r="L812" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Xelajú MC vs Cobán Imperial</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Xelajú MC</t>
+        </is>
+      </c>
+      <c r="D813" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E813" t="inlineStr"/>
+      <c r="F813" t="inlineStr"/>
+      <c r="G813" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H813" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I813" t="n">
+        <v>0</v>
+      </c>
+      <c r="J813" t="n">
+        <v>0</v>
+      </c>
+      <c r="K813" t="n">
+        <v>0</v>
+      </c>
+      <c r="L813" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -37205,7 +37875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37443,6 +38113,25 @@
       </c>
       <c r="E13" t="n">
         <v>49</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>16</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
@@ -37456,7 +38145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37696,6 +38385,216 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>5</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>11</v>
+      </c>
+      <c r="D15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" t="n">
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>66.7</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>value_alert</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fase 4: cierre de resultados 2026-09-12
</commit_message>
<xml_diff>
--- a/data/estadisticas.xlsx
+++ b/data/estadisticas.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L813"/>
+  <dimension ref="A1:L869"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37117,8 +37117,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E798" t="inlineStr"/>
-      <c r="F798" t="inlineStr"/>
       <c r="G798" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -37165,8 +37163,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E799" t="inlineStr"/>
-      <c r="F799" t="inlineStr"/>
       <c r="G799" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -37213,8 +37209,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E800" t="inlineStr"/>
-      <c r="F800" t="inlineStr"/>
       <c r="G800" t="inlineStr">
         <is>
           <t>3-1</t>
@@ -37261,8 +37255,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E801" t="inlineStr"/>
-      <c r="F801" t="inlineStr"/>
       <c r="G801" t="inlineStr">
         <is>
           <t>5-0</t>
@@ -37309,8 +37301,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E802" t="inlineStr"/>
-      <c r="F802" t="inlineStr"/>
       <c r="G802" t="inlineStr">
         <is>
           <t>4-1</t>
@@ -37357,8 +37347,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E803" t="inlineStr"/>
-      <c r="F803" t="inlineStr"/>
       <c r="G803" t="inlineStr">
         <is>
           <t>4-0</t>
@@ -37405,8 +37393,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E804" t="inlineStr"/>
-      <c r="F804" t="inlineStr"/>
       <c r="G804" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -37453,8 +37439,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E805" t="inlineStr"/>
-      <c r="F805" t="inlineStr"/>
       <c r="G805" t="inlineStr">
         <is>
           <t>2-1</t>
@@ -37501,8 +37485,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E806" t="inlineStr"/>
-      <c r="F806" t="inlineStr"/>
       <c r="G806" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -37549,8 +37531,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E807" t="inlineStr"/>
-      <c r="F807" t="inlineStr"/>
       <c r="G807" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -37597,8 +37577,6 @@
           <t>Visitante</t>
         </is>
       </c>
-      <c r="E808" t="inlineStr"/>
-      <c r="F808" t="inlineStr"/>
       <c r="G808" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -37645,8 +37623,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E809" t="inlineStr"/>
-      <c r="F809" t="inlineStr"/>
       <c r="G809" t="inlineStr">
         <is>
           <t>1-2</t>
@@ -37693,8 +37669,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E810" t="inlineStr"/>
-      <c r="F810" t="inlineStr"/>
       <c r="G810" t="inlineStr">
         <is>
           <t>2-0</t>
@@ -37741,8 +37715,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E811" t="inlineStr"/>
-      <c r="F811" t="inlineStr"/>
       <c r="G811" t="inlineStr">
         <is>
           <t>1-1</t>
@@ -37789,8 +37761,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E812" t="inlineStr"/>
-      <c r="F812" t="inlineStr"/>
       <c r="G812" t="inlineStr">
         <is>
           <t>0-2</t>
@@ -37837,8 +37807,6 @@
           <t>Local</t>
         </is>
       </c>
-      <c r="E813" t="inlineStr"/>
-      <c r="F813" t="inlineStr"/>
       <c r="G813" t="inlineStr">
         <is>
           <t>0-0</t>
@@ -37859,6 +37827,2694 @@
         <v>0</v>
       </c>
       <c r="L813" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Kyoto Sanga vs Kashiwa Reysol</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Kashiwa Reysol</t>
+        </is>
+      </c>
+      <c r="D814" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E814" t="inlineStr"/>
+      <c r="F814" t="inlineStr"/>
+      <c r="G814" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H814" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I814" t="n">
+        <v>0</v>
+      </c>
+      <c r="J814" t="n">
+        <v>0</v>
+      </c>
+      <c r="K814" t="n">
+        <v>0</v>
+      </c>
+      <c r="L814" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Vissel Kobe vs Kashima Antlers</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Kashima Antlers</t>
+        </is>
+      </c>
+      <c r="D815" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E815" t="inlineStr"/>
+      <c r="F815" t="inlineStr"/>
+      <c r="G815" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H815" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I815" t="n">
+        <v>0</v>
+      </c>
+      <c r="J815" t="n">
+        <v>0</v>
+      </c>
+      <c r="K815" t="n">
+        <v>0</v>
+      </c>
+      <c r="L815" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Al Qadsiah vs Al Ettifaq</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Al Qadsiah</t>
+        </is>
+      </c>
+      <c r="D816" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E816" t="inlineStr"/>
+      <c r="F816" t="inlineStr"/>
+      <c r="G816" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="H816" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I816" t="n">
+        <v>1</v>
+      </c>
+      <c r="J816" t="n">
+        <v>0</v>
+      </c>
+      <c r="K816" t="n">
+        <v>0</v>
+      </c>
+      <c r="L816" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Al Faisaly vs Al Ittihad</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Al Ittihad</t>
+        </is>
+      </c>
+      <c r="D817" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E817" t="inlineStr"/>
+      <c r="F817" t="inlineStr"/>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I817" t="n">
+        <v>3</v>
+      </c>
+      <c r="J817" t="n">
+        <v>0</v>
+      </c>
+      <c r="K817" t="n">
+        <v>0</v>
+      </c>
+      <c r="L817" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>SV Darmstadt 98 vs Arminia Bielefeld</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Arminia Bielefeld</t>
+        </is>
+      </c>
+      <c r="D818" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr"/>
+      <c r="F818" t="inlineStr"/>
+      <c r="G818" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H818" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I818" t="n">
+        <v>1</v>
+      </c>
+      <c r="J818" t="n">
+        <v>0</v>
+      </c>
+      <c r="K818" t="n">
+        <v>0</v>
+      </c>
+      <c r="L818" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>F.C. København vs AC Horsens</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>F.C. København</t>
+        </is>
+      </c>
+      <c r="D819" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E819" t="inlineStr"/>
+      <c r="F819" t="inlineStr"/>
+      <c r="G819" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H819" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I819" t="n">
+        <v>0</v>
+      </c>
+      <c r="J819" t="n">
+        <v>0</v>
+      </c>
+      <c r="K819" t="n">
+        <v>0</v>
+      </c>
+      <c r="L819" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>BK Häcken vs Mjällby AIF</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>BK Häcken</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E820" t="inlineStr"/>
+      <c r="F820" t="inlineStr"/>
+      <c r="G820" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H820" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I820" t="n">
+        <v>4</v>
+      </c>
+      <c r="J820" t="n">
+        <v>0</v>
+      </c>
+      <c r="K820" t="n">
+        <v>0</v>
+      </c>
+      <c r="L820" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Empoli vs Arezzo</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Empoli</t>
+        </is>
+      </c>
+      <c r="D821" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr"/>
+      <c r="F821" t="inlineStr"/>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H821" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I821" t="n">
+        <v>6</v>
+      </c>
+      <c r="J821" t="n">
+        <v>0</v>
+      </c>
+      <c r="K821" t="n">
+        <v>0</v>
+      </c>
+      <c r="L821" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Stellenbosch vs Sekhukhune United FC</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Stellenbosch</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E822" t="inlineStr"/>
+      <c r="F822" t="inlineStr"/>
+      <c r="G822" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H822" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I822" t="n">
+        <v>1</v>
+      </c>
+      <c r="J822" t="n">
+        <v>0</v>
+      </c>
+      <c r="K822" t="n">
+        <v>0</v>
+      </c>
+      <c r="L822" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar vs Willem II</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>AZ Alkmaar</t>
+        </is>
+      </c>
+      <c r="D823" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E823" t="inlineStr"/>
+      <c r="F823" t="inlineStr"/>
+      <c r="G823" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="H823" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I823" t="n">
+        <v>6</v>
+      </c>
+      <c r="J823" t="n">
+        <v>0</v>
+      </c>
+      <c r="K823" t="n">
+        <v>0</v>
+      </c>
+      <c r="L823" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Clermont Foot vs Boulogne</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Clermont Foot</t>
+        </is>
+      </c>
+      <c r="D824" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E824" t="inlineStr"/>
+      <c r="F824" t="inlineStr"/>
+      <c r="G824" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H824" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I824" t="n">
+        <v>5</v>
+      </c>
+      <c r="J824" t="n">
+        <v>0</v>
+      </c>
+      <c r="K824" t="n">
+        <v>0</v>
+      </c>
+      <c r="L824" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Dijon FCO vs Stade Laval</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Dijon FCO</t>
+        </is>
+      </c>
+      <c r="D825" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E825" t="inlineStr"/>
+      <c r="F825" t="inlineStr"/>
+      <c r="G825" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H825" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I825" t="n">
+        <v>5</v>
+      </c>
+      <c r="J825" t="n">
+        <v>0</v>
+      </c>
+      <c r="K825" t="n">
+        <v>0</v>
+      </c>
+      <c r="L825" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Montpellier vs Pau</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Montpellier</t>
+        </is>
+      </c>
+      <c r="D826" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E826" t="inlineStr"/>
+      <c r="F826" t="inlineStr"/>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H826" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I826" t="n">
+        <v>3</v>
+      </c>
+      <c r="J826" t="n">
+        <v>0</v>
+      </c>
+      <c r="K826" t="n">
+        <v>0</v>
+      </c>
+      <c r="L826" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>AS Nancy Lorraine vs Stade de Reims</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Stade de Reims</t>
+        </is>
+      </c>
+      <c r="D827" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E827" t="inlineStr"/>
+      <c r="F827" t="inlineStr"/>
+      <c r="G827" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H827" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I827" t="n">
+        <v>6</v>
+      </c>
+      <c r="J827" t="n">
+        <v>0</v>
+      </c>
+      <c r="K827" t="n">
+        <v>0</v>
+      </c>
+      <c r="L827" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Rodez Aveyron vs Grenoble</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Rodez Aveyron</t>
+        </is>
+      </c>
+      <c r="D828" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E828" t="inlineStr"/>
+      <c r="F828" t="inlineStr"/>
+      <c r="G828" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H828" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I828" t="n">
+        <v>11</v>
+      </c>
+      <c r="J828" t="n">
+        <v>0</v>
+      </c>
+      <c r="K828" t="n">
+        <v>0</v>
+      </c>
+      <c r="L828" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>FC Eindhoven vs FC Dordrecht</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>FC Eindhoven</t>
+        </is>
+      </c>
+      <c r="D829" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr"/>
+      <c r="F829" t="inlineStr"/>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H829" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I829" t="n">
+        <v>3</v>
+      </c>
+      <c r="J829" t="n">
+        <v>0</v>
+      </c>
+      <c r="K829" t="n">
+        <v>0</v>
+      </c>
+      <c r="L829" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>FC Emmen vs De Graafschap</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>FC Emmen</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E830" t="inlineStr"/>
+      <c r="F830" t="inlineStr"/>
+      <c r="G830" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H830" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I830" t="n">
+        <v>4</v>
+      </c>
+      <c r="J830" t="n">
+        <v>0</v>
+      </c>
+      <c r="K830" t="n">
+        <v>0</v>
+      </c>
+      <c r="L830" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Heracles Almelo vs Jong AZ</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Heracles Almelo</t>
+        </is>
+      </c>
+      <c r="D831" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E831" t="inlineStr"/>
+      <c r="F831" t="inlineStr"/>
+      <c r="G831" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="H831" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I831" t="n">
+        <v>8</v>
+      </c>
+      <c r="J831" t="n">
+        <v>0</v>
+      </c>
+      <c r="K831" t="n">
+        <v>0</v>
+      </c>
+      <c r="L831" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Jong Ajax vs RKC Waalwijk</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>RKC Waalwijk</t>
+        </is>
+      </c>
+      <c r="D832" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E832" t="inlineStr"/>
+      <c r="F832" t="inlineStr"/>
+      <c r="G832" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H832" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I832" t="n">
+        <v>7</v>
+      </c>
+      <c r="J832" t="n">
+        <v>0</v>
+      </c>
+      <c r="K832" t="n">
+        <v>0</v>
+      </c>
+      <c r="L832" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>MVV Maastricht vs Almere City</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Almere City</t>
+        </is>
+      </c>
+      <c r="D833" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E833" t="inlineStr"/>
+      <c r="F833" t="inlineStr"/>
+      <c r="G833" t="inlineStr">
+        <is>
+          <t>0-4</t>
+        </is>
+      </c>
+      <c r="H833" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I833" t="n">
+        <v>4</v>
+      </c>
+      <c r="J833" t="n">
+        <v>0</v>
+      </c>
+      <c r="K833" t="n">
+        <v>0</v>
+      </c>
+      <c r="L833" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>NAC Breda vs Jong FC Utrecht</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>NAC Breda</t>
+        </is>
+      </c>
+      <c r="D834" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E834" t="inlineStr"/>
+      <c r="F834" t="inlineStr"/>
+      <c r="G834" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="H834" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I834" t="n">
+        <v>6</v>
+      </c>
+      <c r="J834" t="n">
+        <v>0</v>
+      </c>
+      <c r="K834" t="n">
+        <v>0</v>
+      </c>
+      <c r="L834" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>VVV-Venlo vs TOP Oss</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>VVV-Venlo</t>
+        </is>
+      </c>
+      <c r="D835" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E835" t="inlineStr"/>
+      <c r="F835" t="inlineStr"/>
+      <c r="G835" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H835" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I835" t="n">
+        <v>1</v>
+      </c>
+      <c r="J835" t="n">
+        <v>0</v>
+      </c>
+      <c r="K835" t="n">
+        <v>0</v>
+      </c>
+      <c r="L835" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Al Ahli vs Al Hazem</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Al Ahli</t>
+        </is>
+      </c>
+      <c r="D836" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr"/>
+      <c r="F836" t="inlineStr"/>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H836" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I836" t="n">
+        <v>3</v>
+      </c>
+      <c r="J836" t="n">
+        <v>0</v>
+      </c>
+      <c r="K836" t="n">
+        <v>0</v>
+      </c>
+      <c r="L836" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Helmond Sport vs Jong PSV</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Jong PSV</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E837" t="inlineStr"/>
+      <c r="F837" t="inlineStr"/>
+      <c r="G837" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H837" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I837" t="n">
+        <v>0</v>
+      </c>
+      <c r="J837" t="n">
+        <v>0</v>
+      </c>
+      <c r="K837" t="n">
+        <v>0</v>
+      </c>
+      <c r="L837" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>1. FC Union Berlin vs Schalke 04</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>1. FC Union Berlin</t>
+        </is>
+      </c>
+      <c r="D838" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E838" t="inlineStr"/>
+      <c r="F838" t="inlineStr"/>
+      <c r="G838" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="H838" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I838" t="n">
+        <v>3</v>
+      </c>
+      <c r="J838" t="n">
+        <v>0</v>
+      </c>
+      <c r="K838" t="n">
+        <v>0</v>
+      </c>
+      <c r="L838" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Greenock Morton vs Livingston</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Livingston</t>
+        </is>
+      </c>
+      <c r="D839" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr"/>
+      <c r="F839" t="inlineStr"/>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H839" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I839" t="n">
+        <v>0</v>
+      </c>
+      <c r="J839" t="n">
+        <v>0</v>
+      </c>
+      <c r="K839" t="n">
+        <v>0</v>
+      </c>
+      <c r="L839" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Burgos vs Ceuta</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Burgos</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E840" t="inlineStr"/>
+      <c r="F840" t="inlineStr"/>
+      <c r="G840" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H840" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I840" t="n">
+        <v>3</v>
+      </c>
+      <c r="J840" t="n">
+        <v>0</v>
+      </c>
+      <c r="K840" t="n">
+        <v>0</v>
+      </c>
+      <c r="L840" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Stade Rennais vs Marseille</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>Stade Rennais</t>
+        </is>
+      </c>
+      <c r="D841" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E841" t="inlineStr"/>
+      <c r="F841" t="inlineStr"/>
+      <c r="G841" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H841" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I841" t="n">
+        <v>0</v>
+      </c>
+      <c r="J841" t="n">
+        <v>0</v>
+      </c>
+      <c r="K841" t="n">
+        <v>0</v>
+      </c>
+      <c r="L841" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Venezia vs Fiorentina</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Fiorentina</t>
+        </is>
+      </c>
+      <c r="D842" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E842" t="inlineStr"/>
+      <c r="F842" t="inlineStr"/>
+      <c r="G842" t="inlineStr">
+        <is>
+          <t>2-4</t>
+        </is>
+      </c>
+      <c r="H842" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I842" t="n">
+        <v>2</v>
+      </c>
+      <c r="J842" t="n">
+        <v>0</v>
+      </c>
+      <c r="K842" t="n">
+        <v>0</v>
+      </c>
+      <c r="L842" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>KV Mechelen vs Anderlecht</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Anderlecht</t>
+        </is>
+      </c>
+      <c r="D843" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr"/>
+      <c r="F843" t="inlineStr"/>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H843" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I843" t="n">
+        <v>5</v>
+      </c>
+      <c r="J843" t="n">
+        <v>0</v>
+      </c>
+      <c r="K843" t="n">
+        <v>0</v>
+      </c>
+      <c r="L843" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Kidderminster Harriers vs Hartlepool United</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Kidderminster Harriers</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E844" t="inlineStr"/>
+      <c r="F844" t="inlineStr"/>
+      <c r="G844" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H844" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I844" t="n">
+        <v>1</v>
+      </c>
+      <c r="J844" t="n">
+        <v>0</v>
+      </c>
+      <c r="K844" t="n">
+        <v>0</v>
+      </c>
+      <c r="L844" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Stenhousemuir vs Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Heart of Midlothian</t>
+        </is>
+      </c>
+      <c r="D845" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E845" t="inlineStr"/>
+      <c r="F845" t="inlineStr"/>
+      <c r="G845" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H845" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I845" t="n">
+        <v>0</v>
+      </c>
+      <c r="J845" t="n">
+        <v>0</v>
+      </c>
+      <c r="K845" t="n">
+        <v>0</v>
+      </c>
+      <c r="L845" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Sevilla vs Valencia</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="D846" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr"/>
+      <c r="F846" t="inlineStr"/>
+      <c r="G846" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H846" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I846" t="n">
+        <v>7</v>
+      </c>
+      <c r="J846" t="n">
+        <v>0</v>
+      </c>
+      <c r="K846" t="n">
+        <v>0</v>
+      </c>
+      <c r="L846" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>West Ham United vs Wrexham</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>West Ham United</t>
+        </is>
+      </c>
+      <c r="D847" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E847" t="inlineStr"/>
+      <c r="F847" t="inlineStr"/>
+      <c r="G847" t="inlineStr">
+        <is>
+          <t>6-0</t>
+        </is>
+      </c>
+      <c r="H847" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I847" t="n">
+        <v>3</v>
+      </c>
+      <c r="J847" t="n">
+        <v>0</v>
+      </c>
+      <c r="K847" t="n">
+        <v>0</v>
+      </c>
+      <c r="L847" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Pisa vs Virtus Entella</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Pisa</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E848" t="inlineStr"/>
+      <c r="F848" t="inlineStr"/>
+      <c r="G848" t="inlineStr">
+        <is>
+          <t>1-4</t>
+        </is>
+      </c>
+      <c r="H848" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I848" t="n">
+        <v>1</v>
+      </c>
+      <c r="J848" t="n">
+        <v>0</v>
+      </c>
+      <c r="K848" t="n">
+        <v>0</v>
+      </c>
+      <c r="L848" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Sportivo Ameliano vs Sportivo San Lorenzo</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Sportivo Ameliano</t>
+        </is>
+      </c>
+      <c r="D849" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E849" t="inlineStr"/>
+      <c r="F849" t="inlineStr"/>
+      <c r="G849" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H849" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I849" t="n">
+        <v>0</v>
+      </c>
+      <c r="J849" t="n">
+        <v>0</v>
+      </c>
+      <c r="K849" t="n">
+        <v>0</v>
+      </c>
+      <c r="L849" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>UTC vs Juan Pablo II</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>UTC</t>
+        </is>
+      </c>
+      <c r="D850" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E850" t="inlineStr"/>
+      <c r="F850" t="inlineStr"/>
+      <c r="G850" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="H850" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I850" t="n">
+        <v>5</v>
+      </c>
+      <c r="J850" t="n">
+        <v>0</v>
+      </c>
+      <c r="K850" t="n">
+        <v>0</v>
+      </c>
+      <c r="L850" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>2 de Mayo vs Libertad</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Libertad</t>
+        </is>
+      </c>
+      <c r="D851" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E851" t="inlineStr"/>
+      <c r="F851" t="inlineStr"/>
+      <c r="G851" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H851" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I851" t="n">
+        <v>1</v>
+      </c>
+      <c r="J851" t="n">
+        <v>0</v>
+      </c>
+      <c r="K851" t="n">
+        <v>0</v>
+      </c>
+      <c r="L851" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Ituzaingó vs Comunicaciones</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Comunicaciones</t>
+        </is>
+      </c>
+      <c r="D852" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E852" t="inlineStr"/>
+      <c r="F852" t="inlineStr"/>
+      <c r="G852" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H852" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I852" t="n">
+        <v>0</v>
+      </c>
+      <c r="J852" t="n">
+        <v>0</v>
+      </c>
+      <c r="K852" t="n">
+        <v>0</v>
+      </c>
+      <c r="L852" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>San Antonio Bulo Bulo vs Aurora</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>San Antonio Bulo Bulo</t>
+        </is>
+      </c>
+      <c r="D853" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E853" t="inlineStr"/>
+      <c r="F853" t="inlineStr"/>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H853" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I853" t="n">
+        <v>0</v>
+      </c>
+      <c r="J853" t="n">
+        <v>0</v>
+      </c>
+      <c r="K853" t="n">
+        <v>0</v>
+      </c>
+      <c r="L853" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Defensa y Justicia vs Gimnasia (Mendoza)</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Defensa y Justicia</t>
+        </is>
+      </c>
+      <c r="D854" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E854" t="inlineStr"/>
+      <c r="F854" t="inlineStr"/>
+      <c r="G854" t="inlineStr">
+        <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="H854" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I854" t="n">
+        <v>0</v>
+      </c>
+      <c r="J854" t="n">
+        <v>0</v>
+      </c>
+      <c r="K854" t="n">
+        <v>0</v>
+      </c>
+      <c r="L854" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Argentino de Merlo vs Real Pilar</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Real Pilar</t>
+        </is>
+      </c>
+      <c r="D855" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E855" t="inlineStr"/>
+      <c r="F855" t="inlineStr"/>
+      <c r="G855" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H855" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I855" t="n">
+        <v>0</v>
+      </c>
+      <c r="J855" t="n">
+        <v>0</v>
+      </c>
+      <c r="K855" t="n">
+        <v>0</v>
+      </c>
+      <c r="L855" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>One Knoxville vs FC Naples</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>One Knoxville</t>
+        </is>
+      </c>
+      <c r="D856" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E856" t="inlineStr"/>
+      <c r="F856" t="inlineStr"/>
+      <c r="G856" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H856" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I856" t="n">
+        <v>0</v>
+      </c>
+      <c r="J856" t="n">
+        <v>0</v>
+      </c>
+      <c r="K856" t="n">
+        <v>0</v>
+      </c>
+      <c r="L856" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Real Potosí vs Oriente Petrolero</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Real Potosí</t>
+        </is>
+      </c>
+      <c r="D857" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr"/>
+      <c r="F857" t="inlineStr"/>
+      <c r="G857" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H857" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I857" t="n">
+        <v>0</v>
+      </c>
+      <c r="J857" t="n">
+        <v>0</v>
+      </c>
+      <c r="K857" t="n">
+        <v>0</v>
+      </c>
+      <c r="L857" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Cusco FC vs Melgar</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>Cusco FC</t>
+        </is>
+      </c>
+      <c r="D858" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E858" t="inlineStr"/>
+      <c r="F858" t="inlineStr"/>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H858" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I858" t="n">
+        <v>2</v>
+      </c>
+      <c r="J858" t="n">
+        <v>0</v>
+      </c>
+      <c r="K858" t="n">
+        <v>0</v>
+      </c>
+      <c r="L858" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Boca Juniors vs Central Córdoba (Santiago del Estero)</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Boca Juniors</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E859" t="inlineStr"/>
+      <c r="F859" t="inlineStr"/>
+      <c r="G859" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I859" t="n">
+        <v>1</v>
+      </c>
+      <c r="J859" t="n">
+        <v>0</v>
+      </c>
+      <c r="K859" t="n">
+        <v>0</v>
+      </c>
+      <c r="L859" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Necaxa vs Puebla</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>Necaxa</t>
+        </is>
+      </c>
+      <c r="D860" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E860" t="inlineStr"/>
+      <c r="F860" t="inlineStr"/>
+      <c r="G860" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H860" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I860" t="n">
+        <v>1</v>
+      </c>
+      <c r="J860" t="n">
+        <v>0</v>
+      </c>
+      <c r="K860" t="n">
+        <v>0</v>
+      </c>
+      <c r="L860" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Gimnasia y Tiro (Salta) vs Tristán Suárez</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Gimnasia y Tiro (Salta)</t>
+        </is>
+      </c>
+      <c r="D861" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr"/>
+      <c r="F861" t="inlineStr"/>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>0-0</t>
+        </is>
+      </c>
+      <c r="H861" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I861" t="n">
+        <v>0</v>
+      </c>
+      <c r="J861" t="n">
+        <v>0</v>
+      </c>
+      <c r="K861" t="n">
+        <v>0</v>
+      </c>
+      <c r="L861" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Correcaminos UAT vs Cancún FC</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Correcaminos UAT</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E862" t="inlineStr"/>
+      <c r="F862" t="inlineStr"/>
+      <c r="G862" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H862" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I862" t="n">
+        <v>0</v>
+      </c>
+      <c r="J862" t="n">
+        <v>0</v>
+      </c>
+      <c r="K862" t="n">
+        <v>0</v>
+      </c>
+      <c r="L862" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>CD Estrella Roja vs Platense</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>CD Estrella Roja</t>
+        </is>
+      </c>
+      <c r="D863" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E863" t="inlineStr"/>
+      <c r="F863" t="inlineStr"/>
+      <c r="G863" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H863" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I863" t="n">
+        <v>0</v>
+      </c>
+      <c r="J863" t="n">
+        <v>0</v>
+      </c>
+      <c r="K863" t="n">
+        <v>0</v>
+      </c>
+      <c r="L863" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Independiente Santa Fe vs Deportes Tolima</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>Independiente Santa Fe</t>
+        </is>
+      </c>
+      <c r="D864" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr"/>
+      <c r="F864" t="inlineStr"/>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+      <c r="H864" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I864" t="n">
+        <v>0</v>
+      </c>
+      <c r="J864" t="n">
+        <v>0</v>
+      </c>
+      <c r="K864" t="n">
+        <v>0</v>
+      </c>
+      <c r="L864" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>New Mexico United vs Indy Eleven</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>New Mexico United</t>
+        </is>
+      </c>
+      <c r="D865" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E865" t="inlineStr"/>
+      <c r="F865" t="inlineStr"/>
+      <c r="G865" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="H865" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I865" t="n">
+        <v>0</v>
+      </c>
+      <c r="J865" t="n">
+        <v>0</v>
+      </c>
+      <c r="K865" t="n">
+        <v>0</v>
+      </c>
+      <c r="L865" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Pérez Zeledón vs AD San Carlos</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Pérez Zeledón</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E866" t="inlineStr"/>
+      <c r="F866" t="inlineStr"/>
+      <c r="G866" t="inlineStr">
+        <is>
+          <t>0-2</t>
+        </is>
+      </c>
+      <c r="H866" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I866" t="n">
+        <v>0</v>
+      </c>
+      <c r="J866" t="n">
+        <v>0</v>
+      </c>
+      <c r="K866" t="n">
+        <v>0</v>
+      </c>
+      <c r="L866" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Colorado Springs Switchbacks FC vs San Antonio FC</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Colorado Springs Switchbacks FC</t>
+        </is>
+      </c>
+      <c r="D867" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E867" t="inlineStr"/>
+      <c r="F867" t="inlineStr"/>
+      <c r="G867" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="H867" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I867" t="n">
+        <v>0</v>
+      </c>
+      <c r="J867" t="n">
+        <v>0</v>
+      </c>
+      <c r="K867" t="n">
+        <v>0</v>
+      </c>
+      <c r="L867" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Atlante vs Pachuca</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Pachuca</t>
+        </is>
+      </c>
+      <c r="D868" t="inlineStr">
+        <is>
+          <t>Visitante</t>
+        </is>
+      </c>
+      <c r="E868" t="inlineStr"/>
+      <c r="F868" t="inlineStr"/>
+      <c r="G868" t="inlineStr">
+        <is>
+          <t>0-3</t>
+        </is>
+      </c>
+      <c r="H868" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="I868" t="n">
+        <v>0</v>
+      </c>
+      <c r="J868" t="n">
+        <v>0</v>
+      </c>
+      <c r="K868" t="n">
+        <v>0</v>
+      </c>
+      <c r="L868" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Tijuana vs Querétaro</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Tijuana</t>
+        </is>
+      </c>
+      <c r="D869" t="inlineStr">
+        <is>
+          <t>Local</t>
+        </is>
+      </c>
+      <c r="E869" t="inlineStr"/>
+      <c r="F869" t="inlineStr"/>
+      <c r="G869" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="H869" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I869" t="n">
+        <v>0</v>
+      </c>
+      <c r="J869" t="n">
+        <v>0</v>
+      </c>
+      <c r="K869" t="n">
+        <v>0</v>
+      </c>
+      <c r="L869" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -37875,7 +40531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38132,6 +40788,25 @@
       </c>
       <c r="E14" t="n">
         <v>16</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>56</v>
+      </c>
+      <c r="C15" t="n">
+        <v>37</v>
+      </c>
+      <c r="D15" t="n">
+        <v>66.09999999999999</v>
+      </c>
+      <c r="E15" t="n">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -38145,7 +40820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -38595,6 +41270,258 @@
         <v>0</v>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>posible_victoria_favorito</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>22</v>
+      </c>
+      <c r="D22" t="n">
+        <v>7</v>
+      </c>
+      <c r="E22" t="n">
+        <v>31.8</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>alerta_1er_tiempo</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>12</v>
+      </c>
+      <c r="D23" t="n">
+        <v>4</v>
+      </c>
+      <c r="E23" t="n">
+        <v>33.3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>fav_domina_no_gana</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>10</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>posible_empate</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>13</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="n">
+        <v>30.8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>no_fav_domina</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>17</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>cuidado_rival_presiona</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>24</v>
+      </c>
+      <c r="D27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" t="n">
+        <v>20.8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>tarjeta_roja</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>gol_de_cierre</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>10</v>
+      </c>
+      <c r="D29" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ampliacion_marcador</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>5</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>siguen_empatados_70</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>value_alert</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>siguen_empatados_22</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>